<commit_message>
:white_circle: Dev v4.1.2: CH4 - Mechanical characteristics
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014BD4DE-8336-4D0C-A759-F9A00D439204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A5EC63-AFA2-44CC-8573-B09467C3AF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -9925,6 +9925,12 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9932,12 +9938,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>

</xml_diff>

<commit_message>
:white_circle: Dev v4.1.11: CH4 - Econominal Analysis
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A5EC63-AFA2-44CC-8573-B09467C3AF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F0B66C-5D1C-4516-B3A5-6BD63BF81B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -9925,12 +9925,6 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9938,6 +9932,12 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>

</xml_diff>

<commit_message>
:white_circle: Dev v4.1.12: CH4 - Technologies (editing)
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F0B66C-5D1C-4516-B3A5-6BD63BF81B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A2FD42-6197-47CD-A315-91FC1DFFAF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -854,12 +854,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0000000"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
+    <numFmt numFmtId="170" formatCode="0.E+00"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1191,7 +1192,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1383,6 +1384,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5873,20 +5877,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25756F58-999A-49F8-9434-550682CD0993}">
   <dimension ref="A5:N59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.26953125" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:13" ht="18.75">
+    <row r="5" spans="1:13" ht="18.5">
       <c r="C5" s="94" t="s">
         <v>151</v>
       </c>
@@ -6400,7 +6404,7 @@
       <c r="M36" s="62"/>
       <c r="N36" s="61"/>
     </row>
-    <row r="37" spans="3:14" ht="18.75">
+    <row r="37" spans="3:14" ht="18.5">
       <c r="C37" s="69"/>
       <c r="D37" s="69"/>
       <c r="E37" s="69"/>
@@ -6600,19 +6604,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F2D825-F3B9-4690-816B-819C9229FE1F}">
   <dimension ref="A2:U57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" ht="18.75">
+    <row r="2" spans="1:21" ht="18.5">
       <c r="C2" s="69"/>
       <c r="D2" s="69"/>
       <c r="E2" s="69"/>
@@ -7289,7 +7293,7 @@
       <c r="O33" s="46"/>
       <c r="P33" s="48"/>
     </row>
-    <row r="34" spans="3:20" ht="18.75">
+    <row r="34" spans="3:20" ht="18.5">
       <c r="C34" s="69"/>
       <c r="D34" s="69"/>
       <c r="E34" s="69"/>
@@ -7658,9 +7662,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC9A626-FE2C-45BC-B5E1-E7D34819B267}">
   <dimension ref="C4:H16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="4" max="4" width="50.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="3:8">
@@ -7808,21 +7812,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:M1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="58.5703125" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" customWidth="1"/>
-    <col min="4" max="4" width="41.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" customWidth="1"/>
+    <col min="2" max="2" width="58.54296875" customWidth="1"/>
+    <col min="3" max="3" width="36.7265625" customWidth="1"/>
+    <col min="4" max="4" width="41.1796875" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
-    <col min="6" max="6" width="58.5703125" customWidth="1"/>
-    <col min="7" max="7" width="36.7109375" customWidth="1"/>
-    <col min="8" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" customWidth="1"/>
-    <col min="13" max="26" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="58.54296875" customWidth="1"/>
+    <col min="7" max="7" width="36.7265625" customWidth="1"/>
+    <col min="8" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" customWidth="1"/>
+    <col min="13" max="26" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13">
+    <row r="1" spans="2:13" ht="14.5">
       <c r="B1" s="97" t="s">
         <v>11</v>
       </c>
@@ -7832,7 +7836,7 @@
       <c r="F1" s="98"/>
       <c r="G1" s="99"/>
     </row>
-    <row r="2" spans="2:13">
+    <row r="2" spans="2:13" ht="14.5">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -7841,7 +7845,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:13">
+    <row r="3" spans="2:13" ht="14.5">
       <c r="B3" s="100" t="s">
         <v>13</v>
       </c>
@@ -7851,7 +7855,7 @@
       </c>
       <c r="G3" s="96"/>
     </row>
-    <row r="4" spans="2:13">
+    <row r="4" spans="2:13" ht="14.5">
       <c r="B4" s="95" t="s">
         <v>1</v>
       </c>
@@ -7861,7 +7865,7 @@
       </c>
       <c r="G4" s="96"/>
     </row>
-    <row r="5" spans="2:13">
+    <row r="5" spans="2:13" ht="14.5">
       <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
@@ -7877,7 +7881,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:13">
+    <row r="6" spans="2:13" ht="14.5">
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
@@ -7903,7 +7907,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:13">
+    <row r="7" spans="2:13" ht="14.5">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
@@ -7933,7 +7937,7 @@
         <v>6.9999999999999951E-2</v>
       </c>
     </row>
-    <row r="8" spans="2:13">
+    <row r="8" spans="2:13" ht="14.5">
       <c r="J8" s="1">
         <v>12</v>
       </c>
@@ -7949,7 +7953,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="9" spans="2:13">
+    <row r="9" spans="2:13" ht="14.5">
       <c r="B9" s="95" t="s">
         <v>4</v>
       </c>
@@ -7973,7 +7977,7 @@
         <v>0.33999999999999997</v>
       </c>
     </row>
-    <row r="10" spans="2:13">
+    <row r="10" spans="2:13" ht="14.5">
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
@@ -8003,7 +8007,7 @@
         <v>0.42000000000000004</v>
       </c>
     </row>
-    <row r="11" spans="2:13">
+    <row r="11" spans="2:13" ht="14.5">
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -8033,7 +8037,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="12" spans="2:13">
+    <row r="12" spans="2:13" ht="14.5">
       <c r="B12" s="7" t="s">
         <v>6</v>
       </c>
@@ -8061,7 +8065,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="13" spans="2:13">
+    <row r="13" spans="2:13" ht="14.5">
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
@@ -8090,7 +8094,7 @@
         <v>0.58000000000000007</v>
       </c>
     </row>
-    <row r="14" spans="2:13">
+    <row r="14" spans="2:13" ht="14.5">
       <c r="F14" s="1" t="s">
         <v>20</v>
       </c>
@@ -8113,7 +8117,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="15" spans="2:13">
+    <row r="15" spans="2:13" ht="14.5">
       <c r="B15" s="95" t="s">
         <v>7</v>
       </c>
@@ -8140,7 +8144,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="16" spans="2:13">
+    <row r="16" spans="2:13" ht="14.5">
       <c r="B16" s="1" t="s">
         <v>8</v>
       </c>
@@ -8162,7 +8166,7 @@
         <v>0.66999999999999993</v>
       </c>
     </row>
-    <row r="17" spans="2:13">
+    <row r="17" spans="2:13" ht="14.5">
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -8186,7 +8190,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="18" spans="2:13">
+    <row r="18" spans="2:13" ht="14.5">
       <c r="B18" s="6" t="s">
         <v>10</v>
       </c>
@@ -8210,7 +8214,7 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="19" spans="2:13">
+    <row r="19" spans="2:13" ht="14.5">
       <c r="B19" s="1" t="s">
         <v>21</v>
       </c>
@@ -8218,7 +8222,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="2:13">
+    <row r="20" spans="2:13" ht="14.5">
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
@@ -9925,6 +9929,12 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9932,12 +9942,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -9952,26 +9956,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="C3:P1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" customWidth="1"/>
-    <col min="4" max="4" width="30.140625" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="59.140625" customWidth="1"/>
-    <col min="7" max="7" width="31.42578125" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="59.140625" customWidth="1"/>
-    <col min="10" max="10" width="31.42578125" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="23.85546875" customWidth="1"/>
-    <col min="13" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="17.85546875" customWidth="1"/>
-    <col min="16" max="16" width="20.140625" customWidth="1"/>
-    <col min="17" max="26" width="11.42578125" customWidth="1"/>
+    <col min="1" max="2" width="11.453125" customWidth="1"/>
+    <col min="3" max="3" width="58.54296875" customWidth="1"/>
+    <col min="4" max="4" width="30.1796875" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="59.1796875" customWidth="1"/>
+    <col min="7" max="7" width="31.453125" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" customWidth="1"/>
+    <col min="9" max="9" width="59.1796875" customWidth="1"/>
+    <col min="10" max="10" width="31.453125" customWidth="1"/>
+    <col min="11" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="23.81640625" customWidth="1"/>
+    <col min="13" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="17.81640625" customWidth="1"/>
+    <col min="16" max="16" width="20.1796875" customWidth="1"/>
+    <col min="17" max="26" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:16" ht="15.75">
+    <row r="3" spans="3:16" ht="16">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -9992,7 +9996,7 @@
       </c>
       <c r="L3" s="93"/>
     </row>
-    <row r="4" spans="3:16">
+    <row r="4" spans="3:16" ht="14.5">
       <c r="C4" s="1" t="s">
         <v>73</v>
       </c>
@@ -10017,7 +10021,7 @@
       <c r="O4" s="17"/>
       <c r="P4" s="18"/>
     </row>
-    <row r="5" spans="3:16">
+    <row r="5" spans="3:16" ht="14.5">
       <c r="C5" s="1" t="s">
         <v>75</v>
       </c>
@@ -10042,14 +10046,14 @@
       <c r="O5" s="16"/>
       <c r="P5" s="19"/>
     </row>
-    <row r="6" spans="3:16">
+    <row r="6" spans="3:16" ht="14.5">
       <c r="L6" s="3"/>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
       <c r="P6" s="19"/>
     </row>
-    <row r="7" spans="3:16">
+    <row r="7" spans="3:16" ht="14.5">
       <c r="C7" s="1" t="s">
         <v>77</v>
       </c>
@@ -10077,7 +10081,7 @@
       <c r="O7" s="22"/>
       <c r="P7" s="19"/>
     </row>
-    <row r="8" spans="3:16">
+    <row r="8" spans="3:16" ht="14.5">
       <c r="C8" s="1" t="s">
         <v>118</v>
       </c>
@@ -10103,7 +10107,7 @@
       <c r="O8" s="24"/>
       <c r="P8" s="19"/>
     </row>
-    <row r="9" spans="3:16">
+    <row r="9" spans="3:16" ht="14.5">
       <c r="C9" s="1" t="s">
         <v>119</v>
       </c>
@@ -10131,7 +10135,7 @@
       <c r="O9" s="16"/>
       <c r="P9" s="19"/>
     </row>
-    <row r="10" spans="3:16">
+    <row r="10" spans="3:16" ht="14.5">
       <c r="C10" s="1" t="s">
         <v>84</v>
       </c>
@@ -10150,7 +10154,7 @@
       <c r="O10" s="3"/>
       <c r="P10" s="19"/>
     </row>
-    <row r="12" spans="3:16">
+    <row r="12" spans="3:16" ht="14.5">
       <c r="C12" s="1" t="s">
         <v>86</v>
       </c>
@@ -10164,7 +10168,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="13" spans="3:16">
+    <row r="13" spans="3:16" ht="14.5">
       <c r="C13" s="1" t="s">
         <v>88</v>
       </c>
@@ -10178,7 +10182,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="3:16">
+    <row r="14" spans="3:16" ht="14.5">
       <c r="C14" s="1" t="s">
         <v>90</v>
       </c>
@@ -10192,7 +10196,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="3:16">
+    <row r="15" spans="3:16" ht="14.5">
       <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
@@ -10215,7 +10219,7 @@
         <v>4.2588727636363641</v>
       </c>
     </row>
-    <row r="19" spans="3:10">
+    <row r="19" spans="3:10" ht="14.5">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -10226,7 +10230,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:10">
+    <row r="20" spans="3:10" ht="14.5">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -10494,7 +10498,7 @@
       <c r="C33" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="111">
         <f>D15/1000</f>
         <v>4.8999999999999998E-4</v>
       </c>
@@ -10558,42 +10562,46 @@
       </c>
     </row>
     <row r="37" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="109">
         <v>1</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="E37" s="110"/>
+      <c r="F37" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="G37" s="1">
+      <c r="G37" s="109">
         <v>1</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="H37" s="110"/>
+      <c r="I37" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="109">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="109" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="109">
         <v>3</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="E38" s="110"/>
+      <c r="F38" s="109" t="s">
         <v>55</v>
       </c>
-      <c r="G38" s="1">
+      <c r="G38" s="109">
         <v>3</v>
       </c>
-      <c r="I38" s="1" t="s">
+      <c r="H38" s="110"/>
+      <c r="I38" s="109" t="s">
         <v>55</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="109">
         <v>3</v>
       </c>
     </row>
@@ -11850,36 +11858,36 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="C2:X1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" customWidth="1"/>
-    <col min="4" max="4" width="30.140625" customWidth="1"/>
-    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="1" max="2" width="11.453125" customWidth="1"/>
+    <col min="3" max="3" width="58.54296875" customWidth="1"/>
+    <col min="4" max="4" width="30.1796875" customWidth="1"/>
+    <col min="5" max="6" width="11.453125" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="10" width="11.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.453125" customWidth="1"/>
+    <col min="9" max="10" width="11.453125" customWidth="1"/>
     <col min="11" max="11" width="59" customWidth="1"/>
-    <col min="12" max="12" width="13.42578125" customWidth="1"/>
-    <col min="13" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="26.5703125" customWidth="1"/>
-    <col min="16" max="17" width="11.85546875" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" customWidth="1"/>
-    <col min="19" max="19" width="11.42578125" customWidth="1"/>
-    <col min="20" max="20" width="22.5703125" customWidth="1"/>
-    <col min="21" max="23" width="11.42578125" customWidth="1"/>
-    <col min="24" max="24" width="14.140625" customWidth="1"/>
-    <col min="25" max="33" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="13.453125" customWidth="1"/>
+    <col min="13" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="26.54296875" customWidth="1"/>
+    <col min="16" max="17" width="11.81640625" customWidth="1"/>
+    <col min="18" max="18" width="16.7265625" customWidth="1"/>
+    <col min="19" max="19" width="11.453125" customWidth="1"/>
+    <col min="20" max="20" width="22.54296875" customWidth="1"/>
+    <col min="21" max="23" width="11.453125" customWidth="1"/>
+    <col min="24" max="24" width="14.1796875" customWidth="1"/>
+    <col min="25" max="33" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:24">
+    <row r="2" spans="3:24" ht="14.5">
       <c r="T2" s="16"/>
       <c r="U2" s="17"/>
       <c r="V2" s="17"/>
       <c r="W2" s="17"/>
       <c r="X2" s="18"/>
     </row>
-    <row r="3" spans="3:24">
+    <row r="3" spans="3:24" ht="14.5">
       <c r="C3" s="5" t="s">
         <v>66</v>
       </c>
@@ -11908,7 +11916,7 @@
       <c r="W3" s="16"/>
       <c r="X3" s="19"/>
     </row>
-    <row r="4" spans="3:24">
+    <row r="4" spans="3:24" ht="14.5">
       <c r="C4" s="5" t="s">
         <v>73</v>
       </c>
@@ -11937,7 +11945,7 @@
       <c r="W4" s="16"/>
       <c r="X4" s="19"/>
     </row>
-    <row r="5" spans="3:24">
+    <row r="5" spans="3:24" ht="14.5">
       <c r="C5" s="3" t="s">
         <v>75</v>
       </c>
@@ -11966,7 +11974,7 @@
       <c r="W5" s="22"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="3:24">
+    <row r="6" spans="3:24" ht="14.5">
       <c r="O6" s="16"/>
       <c r="P6" s="21"/>
       <c r="Q6" s="21"/>
@@ -11977,7 +11985,7 @@
       <c r="W6" s="24"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="3:24">
+    <row r="7" spans="3:24" ht="14.5">
       <c r="C7" s="1" t="s">
         <v>77</v>
       </c>
@@ -12007,7 +12015,7 @@
       <c r="W7" s="16"/>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="3:24">
+    <row r="8" spans="3:24" ht="14.5">
       <c r="C8" s="1" t="s">
         <v>79</v>
       </c>
@@ -12031,7 +12039,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
     </row>
-    <row r="9" spans="3:24">
+    <row r="9" spans="3:24" ht="14.5">
       <c r="C9" s="1" t="s">
         <v>81</v>
       </c>
@@ -12039,7 +12047,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="3:24">
+    <row r="10" spans="3:24" ht="14.5">
       <c r="C10" s="1" t="s">
         <v>82</v>
       </c>
@@ -12048,7 +12056,7 @@
         <v>87.3</v>
       </c>
     </row>
-    <row r="11" spans="3:24">
+    <row r="11" spans="3:24" ht="14.5">
       <c r="C11" s="1" t="s">
         <v>83</v>
       </c>
@@ -12073,7 +12081,7 @@
       </c>
       <c r="P11" s="96"/>
     </row>
-    <row r="12" spans="3:24">
+    <row r="12" spans="3:24" ht="14.5">
       <c r="C12" s="1" t="s">
         <v>86</v>
       </c>
@@ -12099,7 +12107,7 @@
         <v>5957</v>
       </c>
     </row>
-    <row r="13" spans="3:24">
+    <row r="13" spans="3:24" ht="14.5">
       <c r="C13" s="1" t="s">
         <v>88</v>
       </c>
@@ -12125,7 +12133,7 @@
         <v>2286</v>
       </c>
     </row>
-    <row r="14" spans="3:24">
+    <row r="14" spans="3:24" ht="14.5">
       <c r="C14" s="1" t="s">
         <v>90</v>
       </c>
@@ -12151,7 +12159,7 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="15" spans="3:24">
+    <row r="15" spans="3:24" ht="14.5">
       <c r="C15" s="1" t="s">
         <v>92</v>
       </c>
@@ -12181,7 +12189,7 @@
         <v>33962548788</v>
       </c>
     </row>
-    <row r="16" spans="3:24">
+    <row r="16" spans="3:24" ht="14.5">
       <c r="O16" s="16" t="s">
         <v>95</v>
       </c>
@@ -12189,7 +12197,7 @@
         <v>33.963000000000001</v>
       </c>
     </row>
-    <row r="17" spans="3:17">
+    <row r="17" spans="3:17" ht="14.5">
       <c r="O17" s="17" t="s">
         <v>96</v>
       </c>
@@ -12197,7 +12205,7 @@
         <v>33963</v>
       </c>
     </row>
-    <row r="18" spans="3:17">
+    <row r="18" spans="3:17" ht="14.5">
       <c r="O18" s="17" t="s">
         <v>97</v>
       </c>
@@ -12205,7 +12213,7 @@
         <v>13750</v>
       </c>
     </row>
-    <row r="19" spans="3:17">
+    <row r="19" spans="3:17" ht="14.5">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -12216,7 +12224,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:17">
+    <row r="20" spans="3:17" ht="14.5">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -13896,33 +13904,33 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="C2:X1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" customWidth="1"/>
-    <col min="4" max="4" width="30.140625" customWidth="1"/>
-    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="1" max="2" width="11.453125" customWidth="1"/>
+    <col min="3" max="3" width="58.54296875" customWidth="1"/>
+    <col min="4" max="4" width="30.1796875" customWidth="1"/>
+    <col min="5" max="6" width="11.453125" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="10" width="11.42578125" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" customWidth="1"/>
+    <col min="9" max="10" width="11.453125" customWidth="1"/>
     <col min="11" max="11" width="59" customWidth="1"/>
-    <col min="12" max="12" width="24.5703125" customWidth="1"/>
-    <col min="13" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="22.5703125" customWidth="1"/>
-    <col min="16" max="17" width="11.85546875" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" customWidth="1"/>
-    <col min="19" max="19" width="11.42578125" customWidth="1"/>
-    <col min="20" max="20" width="21.42578125" customWidth="1"/>
-    <col min="21" max="22" width="11.42578125" customWidth="1"/>
-    <col min="23" max="23" width="12.28515625" customWidth="1"/>
-    <col min="24" max="24" width="14.7109375" customWidth="1"/>
-    <col min="25" max="32" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="24.54296875" customWidth="1"/>
+    <col min="13" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="22.54296875" customWidth="1"/>
+    <col min="16" max="17" width="11.81640625" customWidth="1"/>
+    <col min="18" max="18" width="16.7265625" customWidth="1"/>
+    <col min="19" max="19" width="11.453125" customWidth="1"/>
+    <col min="20" max="20" width="21.453125" customWidth="1"/>
+    <col min="21" max="22" width="11.453125" customWidth="1"/>
+    <col min="23" max="23" width="12.26953125" customWidth="1"/>
+    <col min="24" max="24" width="14.7265625" customWidth="1"/>
+    <col min="25" max="32" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:24" ht="15.75">
+    <row r="2" spans="3:24" ht="16">
       <c r="T2" s="93"/>
     </row>
-    <row r="3" spans="3:24">
+    <row r="3" spans="3:24" ht="14.5">
       <c r="C3" s="5" t="s">
         <v>66</v>
       </c>
@@ -13951,7 +13959,7 @@
       <c r="W3" s="17"/>
       <c r="X3" s="18"/>
     </row>
-    <row r="4" spans="3:24">
+    <row r="4" spans="3:24" ht="14.5">
       <c r="C4" s="5" t="s">
         <v>73</v>
       </c>
@@ -13980,7 +13988,7 @@
       <c r="W4" s="3"/>
       <c r="X4" s="19"/>
     </row>
-    <row r="5" spans="3:24">
+    <row r="5" spans="3:24" ht="14.5">
       <c r="C5" s="3" t="s">
         <v>75</v>
       </c>
@@ -14009,7 +14017,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="3:24">
+    <row r="6" spans="3:24" ht="14.5">
       <c r="K6" s="1" t="s">
         <v>119</v>
       </c>
@@ -14027,7 +14035,7 @@
       <c r="W6" s="20"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="3:24">
+    <row r="7" spans="3:24" ht="14.5">
       <c r="C7" s="1" t="s">
         <v>119</v>
       </c>
@@ -14057,7 +14065,7 @@
       <c r="W7" s="21"/>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="3:24">
+    <row r="8" spans="3:24" ht="14.5">
       <c r="C8" s="1" t="s">
         <v>118</v>
       </c>
@@ -14086,7 +14094,7 @@
       <c r="W8" s="3"/>
       <c r="X8" s="19"/>
     </row>
-    <row r="9" spans="3:24">
+    <row r="9" spans="3:24" ht="14.5">
       <c r="C9" s="1" t="s">
         <v>77</v>
       </c>
@@ -14102,7 +14110,7 @@
         <v>28.000000000000007</v>
       </c>
     </row>
-    <row r="10" spans="3:24">
+    <row r="10" spans="3:24" ht="14.5">
       <c r="C10" s="1" t="s">
         <v>84</v>
       </c>
@@ -14117,7 +14125,7 @@
         <v>3.3600000000000005E-2</v>
       </c>
     </row>
-    <row r="11" spans="3:24">
+    <row r="11" spans="3:24" ht="14.5">
       <c r="K11" s="1" t="s">
         <v>84</v>
       </c>
@@ -14125,7 +14133,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="12" spans="3:24">
+    <row r="12" spans="3:24" ht="14.5">
       <c r="C12" s="1" t="s">
         <v>134</v>
       </c>
@@ -14146,7 +14154,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="13" spans="3:24">
+    <row r="13" spans="3:24" ht="14.5">
       <c r="C13" s="1" t="s">
         <v>136</v>
       </c>
@@ -14166,7 +14174,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="3:24">
+    <row r="15" spans="3:24" ht="14.5">
       <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
@@ -14189,7 +14197,7 @@
         <v>1.69100936968451E-2</v>
       </c>
     </row>
-    <row r="19" spans="3:12">
+    <row r="19" spans="3:12" ht="14.5">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -14200,7 +14208,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:12">
+    <row r="20" spans="3:12" ht="14.5">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -15851,35 +15859,35 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="C3:AJ1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="3" width="25.42578125" customWidth="1"/>
-    <col min="4" max="5" width="10.5703125" customWidth="1"/>
+    <col min="1" max="2" width="10.54296875" customWidth="1"/>
+    <col min="3" max="3" width="25.453125" customWidth="1"/>
+    <col min="4" max="5" width="10.54296875" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="10" width="10.5703125" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="14.5703125" customWidth="1"/>
-    <col min="13" max="13" width="15.5703125" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
-    <col min="15" max="15" width="14.5703125" customWidth="1"/>
-    <col min="16" max="18" width="10.5703125" customWidth="1"/>
-    <col min="19" max="19" width="22.7109375" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="10.54296875" customWidth="1"/>
+    <col min="11" max="11" width="22.7265625" customWidth="1"/>
+    <col min="12" max="12" width="14.54296875" customWidth="1"/>
+    <col min="13" max="13" width="15.54296875" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" customWidth="1"/>
+    <col min="15" max="15" width="14.54296875" customWidth="1"/>
+    <col min="16" max="18" width="10.54296875" customWidth="1"/>
+    <col min="19" max="19" width="22.7265625" customWidth="1"/>
+    <col min="20" max="20" width="10.54296875" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="13" customWidth="1"/>
-    <col min="24" max="26" width="10.5703125" customWidth="1"/>
-    <col min="27" max="27" width="22.7109375" customWidth="1"/>
-    <col min="28" max="28" width="8.28515625" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" customWidth="1"/>
-    <col min="30" max="30" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.28515625" customWidth="1"/>
-    <col min="32" max="32" width="10.5703125" customWidth="1"/>
-    <col min="33" max="33" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" customWidth="1"/>
+    <col min="24" max="26" width="10.54296875" customWidth="1"/>
+    <col min="27" max="27" width="22.7265625" customWidth="1"/>
+    <col min="28" max="28" width="8.26953125" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" customWidth="1"/>
+    <col min="30" max="30" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.26953125" customWidth="1"/>
+    <col min="32" max="32" width="10.54296875" customWidth="1"/>
+    <col min="33" max="33" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:36">
+    <row r="3" spans="3:36" ht="14.5">
       <c r="C3" s="104" t="s">
         <v>110</v>
       </c>
@@ -15915,7 +15923,7 @@
       <c r="AI3" s="105"/>
       <c r="AJ3" s="106"/>
     </row>
-    <row r="4" spans="3:36">
+    <row r="4" spans="3:36" ht="14.5">
       <c r="C4" s="35"/>
       <c r="D4" s="36" t="s">
         <v>113</v>
@@ -15979,7 +15987,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="3:36">
+    <row r="5" spans="3:36" ht="14.5">
       <c r="C5" s="35" t="s">
         <v>74</v>
       </c>
@@ -16058,7 +16066,7 @@
         <v>1916.6666666666665</v>
       </c>
     </row>
-    <row r="6" spans="3:36">
+    <row r="6" spans="3:36" ht="14.5">
       <c r="C6" s="35" t="s">
         <v>117</v>
       </c>
@@ -16146,7 +16154,7 @@
         <v>12096.666666666668</v>
       </c>
     </row>
-    <row r="7" spans="3:36">
+    <row r="7" spans="3:36" ht="14.5">
       <c r="C7" s="35" t="s">
         <v>118</v>
       </c>
@@ -16234,7 +16242,7 @@
         <v>20389.349999999999</v>
       </c>
     </row>
-    <row r="8" spans="3:36">
+    <row r="8" spans="3:36" ht="14.5">
       <c r="C8" s="35" t="s">
         <v>92</v>
       </c>
@@ -16322,7 +16330,7 @@
         <v>19.444272973333334</v>
       </c>
     </row>
-    <row r="9" spans="3:36">
+    <row r="9" spans="3:36" ht="14.5">
       <c r="C9" s="35" t="s">
         <v>78</v>
       </c>
@@ -16410,7 +16418,7 @@
         <v>2940.625</v>
       </c>
     </row>
-    <row r="13" spans="3:36">
+    <row r="13" spans="3:36" ht="14.5">
       <c r="C13" s="104" t="s">
         <v>138</v>
       </c>
@@ -16446,7 +16454,7 @@
       <c r="AI13" s="105"/>
       <c r="AJ13" s="106"/>
     </row>
-    <row r="14" spans="3:36">
+    <row r="14" spans="3:36" ht="14.5">
       <c r="C14" s="35"/>
       <c r="D14" s="36" t="s">
         <v>113</v>
@@ -16510,7 +16518,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="3:36">
+    <row r="15" spans="3:36" ht="14.5">
       <c r="C15" s="35" t="s">
         <v>74</v>
       </c>
@@ -16603,7 +16611,7 @@
         <v>0.76666666666666661</v>
       </c>
     </row>
-    <row r="16" spans="3:36">
+    <row r="16" spans="3:36" ht="14.5">
       <c r="C16" s="35" t="s">
         <v>117</v>
       </c>
@@ -16696,7 +16704,7 @@
         <v>0.96043403466984267</v>
       </c>
     </row>
-    <row r="17" spans="3:36">
+    <row r="17" spans="3:36" ht="14.5">
       <c r="C17" s="35" t="s">
         <v>118</v>
       </c>
@@ -16789,7 +16797,7 @@
         <v>0.72741602697126273</v>
       </c>
     </row>
-    <row r="18" spans="3:36">
+    <row r="18" spans="3:36" ht="14.5">
       <c r="C18" s="35" t="s">
         <v>92</v>
       </c>
@@ -16882,7 +16890,7 @@
         <v>0.85406533109231642</v>
       </c>
     </row>
-    <row r="19" spans="3:36">
+    <row r="19" spans="3:36" ht="14.5">
       <c r="C19" s="35" t="s">
         <v>78</v>
       </c>

</xml_diff>

<commit_message>
:white_circle: Dev v4.1.14: CH4 - APPENDIX
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A2FD42-6197-47CD-A315-91FC1DFFAF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F002E81-DAEB-41B4-BDF8-AC072CD8A192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -860,7 +860,7 @@
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0000000"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
-    <numFmt numFmtId="170" formatCode="0.E+00"/>
+    <numFmt numFmtId="169" formatCode="0.E+00"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1192,7 +1192,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1349,6 +1349,7 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="9" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1384,9 +1385,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5891,12 +5889,12 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:13" ht="18.5">
-      <c r="C5" s="94" t="s">
+      <c r="C5" s="95" t="s">
         <v>151</v>
       </c>
-      <c r="D5" s="94"/>
-      <c r="E5" s="94"/>
-      <c r="F5" s="94"/>
+      <c r="D5" s="95"/>
+      <c r="E5" s="95"/>
+      <c r="F5" s="95"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="42" t="s">
@@ -7744,7 +7742,7 @@
         <v>166</v>
       </c>
       <c r="E9">
-        <v>1.02</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="3:8">
@@ -7756,7 +7754,7 @@
       </c>
       <c r="E10" s="51">
         <f>(E4*E8*E9)/(E7*E6*E5)</f>
-        <v>2793.7373490767045</v>
+        <v>2738.958185369318</v>
       </c>
     </row>
     <row r="11" spans="3:8">
@@ -7765,7 +7763,7 @@
       </c>
       <c r="E11" s="78">
         <f>(E8*E9)/(E5*E6*E7)</f>
-        <v>1.9016335227272725</v>
+        <v>1.8643465909090906</v>
       </c>
     </row>
     <row r="13" spans="3:8">
@@ -7801,7 +7799,7 @@
       </c>
       <c r="E16">
         <f>E15*E9*E8</f>
-        <v>2795.4012784090901</v>
+        <v>2740.5894886363631</v>
       </c>
     </row>
   </sheetData>
@@ -7827,14 +7825,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="14.5">
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="2" spans="2:13" ht="14.5">
       <c r="B2" s="1" t="s">
@@ -7846,24 +7844,24 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="14.5">
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="F3" s="100" t="s">
+      <c r="C3" s="97"/>
+      <c r="F3" s="101" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="96"/>
+      <c r="G3" s="97"/>
     </row>
     <row r="4" spans="2:13" ht="14.5">
-      <c r="B4" s="95" t="s">
+      <c r="B4" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="96"/>
-      <c r="F4" s="95" t="s">
+      <c r="C4" s="97"/>
+      <c r="F4" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="96"/>
+      <c r="G4" s="97"/>
     </row>
     <row r="5" spans="2:13" ht="14.5">
       <c r="B5" s="6" t="s">
@@ -7954,14 +7952,14 @@
       </c>
     </row>
     <row r="9" spans="2:13" ht="14.5">
-      <c r="B9" s="95" t="s">
+      <c r="B9" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="96"/>
-      <c r="F9" s="95" t="s">
+      <c r="C9" s="97"/>
+      <c r="F9" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="96"/>
+      <c r="G9" s="97"/>
       <c r="J9" s="1">
         <v>14</v>
       </c>
@@ -8118,10 +8116,10 @@
       </c>
     </row>
     <row r="15" spans="2:13" ht="14.5">
-      <c r="B15" s="95" t="s">
+      <c r="B15" s="96" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="96"/>
+      <c r="C15" s="97"/>
       <c r="F15" s="6" t="s">
         <v>6</v>
       </c>
@@ -8276,14 +8274,14 @@
       </c>
     </row>
     <row r="24" spans="2:13" ht="15.75" customHeight="1">
-      <c r="B24" s="95" t="s">
+      <c r="B24" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="96"/>
-      <c r="F24" s="95" t="s">
+      <c r="C24" s="97"/>
+      <c r="F24" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="96"/>
+      <c r="G24" s="97"/>
       <c r="J24" s="1">
         <v>12</v>
       </c>
@@ -8541,14 +8539,14 @@
       </c>
     </row>
     <row r="35" spans="2:13" ht="15.75" customHeight="1">
-      <c r="B35" s="97" t="s">
+      <c r="B35" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="98"/>
-      <c r="D35" s="98"/>
-      <c r="E35" s="98"/>
-      <c r="F35" s="98"/>
-      <c r="G35" s="99"/>
+      <c r="C35" s="99"/>
+      <c r="D35" s="99"/>
+      <c r="E35" s="99"/>
+      <c r="F35" s="99"/>
+      <c r="G35" s="100"/>
     </row>
     <row r="36" spans="2:13" ht="15.75" customHeight="1">
       <c r="D36" s="1" t="s">
@@ -8750,14 +8748,14 @@
       </c>
     </row>
     <row r="51" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B51" s="97" t="s">
+      <c r="B51" s="98" t="s">
         <v>48</v>
       </c>
-      <c r="C51" s="99"/>
-      <c r="F51" s="97" t="s">
+      <c r="C51" s="100"/>
+      <c r="F51" s="98" t="s">
         <v>49</v>
       </c>
-      <c r="G51" s="99"/>
+      <c r="G51" s="100"/>
     </row>
     <row r="52" spans="2:12" ht="15.75" customHeight="1">
       <c r="B52" s="1" t="s">
@@ -9929,12 +9927,6 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9942,6 +9934,12 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -10498,7 +10496,7 @@
       <c r="C33" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="111">
+      <c r="D33" s="94">
         <f>D15/1000</f>
         <v>4.8999999999999998E-4</v>
       </c>
@@ -10562,46 +10560,42 @@
       </c>
     </row>
     <row r="37" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C37" s="109" t="s">
+      <c r="C37" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="109">
+      <c r="D37" s="1">
         <v>1</v>
       </c>
-      <c r="E37" s="110"/>
-      <c r="F37" s="109" t="s">
+      <c r="F37" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G37" s="109">
+      <c r="G37" s="1">
         <v>1</v>
       </c>
-      <c r="H37" s="110"/>
-      <c r="I37" s="109" t="s">
+      <c r="I37" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="109">
+      <c r="J37" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C38" s="109" t="s">
+      <c r="C38" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="109">
+      <c r="D38" s="1">
         <v>3</v>
       </c>
-      <c r="E38" s="110"/>
-      <c r="F38" s="109" t="s">
+      <c r="F38" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G38" s="109">
+      <c r="G38" s="1">
         <v>3</v>
       </c>
-      <c r="H38" s="110"/>
-      <c r="I38" s="109" t="s">
+      <c r="I38" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="J38" s="109">
+      <c r="J38" s="1">
         <v>3</v>
       </c>
     </row>
@@ -12076,10 +12070,10 @@
       <c r="L11" s="1">
         <v>1920</v>
       </c>
-      <c r="O11" s="101" t="s">
+      <c r="O11" s="102" t="s">
         <v>85</v>
       </c>
-      <c r="P11" s="96"/>
+      <c r="P11" s="97"/>
     </row>
     <row r="12" spans="3:24" ht="14.5">
       <c r="C12" s="1" t="s">
@@ -12243,10 +12237,10 @@
       <c r="L20" s="82">
         <v>750</v>
       </c>
-      <c r="O20" s="100" t="s">
+      <c r="O20" s="101" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="96"/>
+      <c r="P20" s="97"/>
     </row>
     <row r="21" spans="3:17" ht="15.75" customHeight="1">
       <c r="C21" s="1" t="s">
@@ -12355,10 +12349,10 @@
         <f>L23*L22</f>
         <v>38400</v>
       </c>
-      <c r="O24" s="102" t="s">
+      <c r="O24" s="103" t="s">
         <v>102</v>
       </c>
-      <c r="P24" s="96"/>
+      <c r="P24" s="97"/>
     </row>
     <row r="25" spans="3:17" ht="15.75" customHeight="1">
       <c r="C25" s="81" t="s">
@@ -12459,10 +12453,10 @@
         <f>L27*L26</f>
         <v>3650</v>
       </c>
-      <c r="O28" s="103" t="s">
+      <c r="O28" s="104" t="s">
         <v>147</v>
       </c>
-      <c r="P28" s="103"/>
+      <c r="P28" s="104"/>
     </row>
     <row r="29" spans="3:17" ht="15.75" customHeight="1">
       <c r="C29" s="14" t="s">
@@ -15888,40 +15882,40 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:36" ht="14.5">
-      <c r="C3" s="104" t="s">
+      <c r="C3" s="105" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="107"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="108"/>
-      <c r="K3" s="104" t="s">
+      <c r="D3" s="108"/>
+      <c r="E3" s="108"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="109"/>
+      <c r="K3" s="105" t="s">
         <v>65</v>
       </c>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
-      <c r="N3" s="105"/>
-      <c r="O3" s="106"/>
-      <c r="S3" s="104" t="s">
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="107"/>
+      <c r="S3" s="105" t="s">
         <v>121</v>
       </c>
-      <c r="T3" s="105"/>
-      <c r="U3" s="105"/>
-      <c r="V3" s="105"/>
-      <c r="W3" s="106"/>
-      <c r="AA3" s="104" t="s">
+      <c r="T3" s="106"/>
+      <c r="U3" s="106"/>
+      <c r="V3" s="106"/>
+      <c r="W3" s="107"/>
+      <c r="AA3" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="AB3" s="105"/>
-      <c r="AC3" s="105"/>
-      <c r="AD3" s="105"/>
-      <c r="AE3" s="106"/>
-      <c r="AG3" s="104" t="s">
+      <c r="AB3" s="106"/>
+      <c r="AC3" s="106"/>
+      <c r="AD3" s="106"/>
+      <c r="AE3" s="107"/>
+      <c r="AG3" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="AH3" s="105"/>
-      <c r="AI3" s="105"/>
-      <c r="AJ3" s="106"/>
+      <c r="AH3" s="106"/>
+      <c r="AI3" s="106"/>
+      <c r="AJ3" s="107"/>
     </row>
     <row r="4" spans="3:36" ht="14.5">
       <c r="C4" s="35"/>
@@ -16419,40 +16413,40 @@
       </c>
     </row>
     <row r="13" spans="3:36" ht="14.5">
-      <c r="C13" s="104" t="s">
+      <c r="C13" s="105" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="105"/>
-      <c r="E13" s="105"/>
-      <c r="F13" s="105"/>
-      <c r="G13" s="106"/>
-      <c r="K13" s="104" t="s">
+      <c r="D13" s="106"/>
+      <c r="E13" s="106"/>
+      <c r="F13" s="106"/>
+      <c r="G13" s="107"/>
+      <c r="K13" s="105" t="s">
         <v>140</v>
       </c>
-      <c r="L13" s="105"/>
-      <c r="M13" s="105"/>
-      <c r="N13" s="105"/>
-      <c r="O13" s="106"/>
-      <c r="S13" s="104" t="s">
+      <c r="L13" s="106"/>
+      <c r="M13" s="106"/>
+      <c r="N13" s="106"/>
+      <c r="O13" s="107"/>
+      <c r="S13" s="105" t="s">
         <v>139</v>
       </c>
-      <c r="T13" s="105"/>
-      <c r="U13" s="105"/>
-      <c r="V13" s="105"/>
-      <c r="W13" s="106"/>
-      <c r="AA13" s="104" t="s">
+      <c r="T13" s="106"/>
+      <c r="U13" s="106"/>
+      <c r="V13" s="106"/>
+      <c r="W13" s="107"/>
+      <c r="AA13" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="AB13" s="105"/>
-      <c r="AC13" s="105"/>
-      <c r="AD13" s="105"/>
-      <c r="AE13" s="106"/>
-      <c r="AG13" s="104" t="s">
+      <c r="AB13" s="106"/>
+      <c r="AC13" s="106"/>
+      <c r="AD13" s="106"/>
+      <c r="AE13" s="107"/>
+      <c r="AG13" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="AH13" s="105"/>
-      <c r="AI13" s="105"/>
-      <c r="AJ13" s="106"/>
+      <c r="AH13" s="106"/>
+      <c r="AI13" s="106"/>
+      <c r="AJ13" s="107"/>
     </row>
     <row r="14" spans="3:36" ht="14.5">
       <c r="C14" s="35"/>

</xml_diff>

<commit_message>
:white_circle: Dev v4.1.15: CH4 - Radar Plots
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F002E81-DAEB-41B4-BDF8-AC072CD8A192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4B5879-BC75-4816-A9C6-30D58F219F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -311,7 +311,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="181">
   <si>
     <t xml:space="preserve">Nombre </t>
   </si>
@@ -848,6 +848,12 @@
   </si>
   <si>
     <t>Vgenset (L)</t>
+  </si>
+  <si>
+    <t>Life cycles [-]</t>
+  </si>
+  <si>
+    <t>Cells [-]</t>
   </si>
 </sst>
 </file>
@@ -3299,10 +3305,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -3390,10 +3396,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -3481,10 +3487,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -3572,10 +3578,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -3595,21 +3601,6 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>0.4291666666666667</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.33359662081938429</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.38212279811629662</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.44179055316397275</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.73863699435028241</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -3914,10 +3905,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -4005,10 +3996,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -4096,10 +4087,10 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Ciclos de Vida</c:v>
+                  <c:v>Life cycles [-]</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Celdas Totales</c:v>
+                  <c:v>Cells [-]</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Weight [kg]</c:v>
@@ -4119,21 +4110,6 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>0.76666666666666661</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.96043403466984267</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.72741602697126273</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.85406533109231642</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.7974576271186441</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5875,20 +5851,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25756F58-999A-49F8-9434-550682CD0993}">
   <dimension ref="A5:N59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:13" ht="18.5">
+    <row r="5" spans="1:13" ht="18.75">
       <c r="C5" s="95" t="s">
         <v>151</v>
       </c>
@@ -6402,7 +6378,7 @@
       <c r="M36" s="62"/>
       <c r="N36" s="61"/>
     </row>
-    <row r="37" spans="3:14" ht="18.5">
+    <row r="37" spans="3:14" ht="18.75">
       <c r="C37" s="69"/>
       <c r="D37" s="69"/>
       <c r="E37" s="69"/>
@@ -6602,19 +6578,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F2D825-F3B9-4690-816B-819C9229FE1F}">
   <dimension ref="A2:U57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" ht="18.5">
+    <row r="2" spans="1:21" ht="18.75">
       <c r="C2" s="69"/>
       <c r="D2" s="69"/>
       <c r="E2" s="69"/>
@@ -7291,7 +7267,7 @@
       <c r="O33" s="46"/>
       <c r="P33" s="48"/>
     </row>
-    <row r="34" spans="3:20" ht="18.5">
+    <row r="34" spans="3:20" ht="18.75">
       <c r="C34" s="69"/>
       <c r="D34" s="69"/>
       <c r="E34" s="69"/>
@@ -7660,9 +7636,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC9A626-FE2C-45BC-B5E1-E7D34819B267}">
   <dimension ref="C4:H16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="50.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="3:8">
@@ -7810,21 +7786,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:M1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="58.54296875" customWidth="1"/>
-    <col min="3" max="3" width="36.7265625" customWidth="1"/>
-    <col min="4" max="4" width="41.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="58.5703125" customWidth="1"/>
+    <col min="3" max="3" width="36.7109375" customWidth="1"/>
+    <col min="4" max="4" width="41.140625" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
-    <col min="6" max="6" width="58.54296875" customWidth="1"/>
-    <col min="7" max="7" width="36.7265625" customWidth="1"/>
-    <col min="8" max="11" width="11.453125" customWidth="1"/>
-    <col min="12" max="12" width="16.1796875" customWidth="1"/>
-    <col min="13" max="26" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="58.5703125" customWidth="1"/>
+    <col min="7" max="7" width="36.7109375" customWidth="1"/>
+    <col min="8" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="16.140625" customWidth="1"/>
+    <col min="13" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="14.5">
+    <row r="1" spans="2:13">
       <c r="B1" s="98" t="s">
         <v>11</v>
       </c>
@@ -7834,7 +7810,7 @@
       <c r="F1" s="99"/>
       <c r="G1" s="100"/>
     </row>
-    <row r="2" spans="2:13" ht="14.5">
+    <row r="2" spans="2:13">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -7843,7 +7819,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:13" ht="14.5">
+    <row r="3" spans="2:13">
       <c r="B3" s="101" t="s">
         <v>13</v>
       </c>
@@ -7853,7 +7829,7 @@
       </c>
       <c r="G3" s="97"/>
     </row>
-    <row r="4" spans="2:13" ht="14.5">
+    <row r="4" spans="2:13">
       <c r="B4" s="96" t="s">
         <v>1</v>
       </c>
@@ -7863,7 +7839,7 @@
       </c>
       <c r="G4" s="97"/>
     </row>
-    <row r="5" spans="2:13" ht="14.5">
+    <row r="5" spans="2:13">
       <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
@@ -7879,7 +7855,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="14.5">
+    <row r="6" spans="2:13">
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
@@ -7905,7 +7881,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="14.5">
+    <row r="7" spans="2:13">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
@@ -7935,7 +7911,7 @@
         <v>6.9999999999999951E-2</v>
       </c>
     </row>
-    <row r="8" spans="2:13" ht="14.5">
+    <row r="8" spans="2:13">
       <c r="J8" s="1">
         <v>12</v>
       </c>
@@ -7951,7 +7927,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="9" spans="2:13" ht="14.5">
+    <row r="9" spans="2:13">
       <c r="B9" s="96" t="s">
         <v>4</v>
       </c>
@@ -7975,7 +7951,7 @@
         <v>0.33999999999999997</v>
       </c>
     </row>
-    <row r="10" spans="2:13" ht="14.5">
+    <row r="10" spans="2:13">
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
@@ -8005,7 +7981,7 @@
         <v>0.42000000000000004</v>
       </c>
     </row>
-    <row r="11" spans="2:13" ht="14.5">
+    <row r="11" spans="2:13">
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -8035,7 +8011,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="12" spans="2:13" ht="14.5">
+    <row r="12" spans="2:13">
       <c r="B12" s="7" t="s">
         <v>6</v>
       </c>
@@ -8063,7 +8039,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="13" spans="2:13" ht="14.5">
+    <row r="13" spans="2:13">
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
@@ -8092,7 +8068,7 @@
         <v>0.58000000000000007</v>
       </c>
     </row>
-    <row r="14" spans="2:13" ht="14.5">
+    <row r="14" spans="2:13">
       <c r="F14" s="1" t="s">
         <v>20</v>
       </c>
@@ -8115,7 +8091,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="15" spans="2:13" ht="14.5">
+    <row r="15" spans="2:13">
       <c r="B15" s="96" t="s">
         <v>7</v>
       </c>
@@ -8142,7 +8118,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="14.5">
+    <row r="16" spans="2:13">
       <c r="B16" s="1" t="s">
         <v>8</v>
       </c>
@@ -8164,7 +8140,7 @@
         <v>0.66999999999999993</v>
       </c>
     </row>
-    <row r="17" spans="2:13" ht="14.5">
+    <row r="17" spans="2:13">
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -8188,7 +8164,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="18" spans="2:13" ht="14.5">
+    <row r="18" spans="2:13">
       <c r="B18" s="6" t="s">
         <v>10</v>
       </c>
@@ -8212,7 +8188,7 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="19" spans="2:13" ht="14.5">
+    <row r="19" spans="2:13">
       <c r="B19" s="1" t="s">
         <v>21</v>
       </c>
@@ -8220,7 +8196,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="2:13" ht="14.5">
+    <row r="20" spans="2:13">
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
@@ -9927,6 +9903,12 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9934,12 +9916,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -9954,26 +9930,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="C3:P1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.453125" customWidth="1"/>
-    <col min="3" max="3" width="58.54296875" customWidth="1"/>
-    <col min="4" max="4" width="30.1796875" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" customWidth="1"/>
-    <col min="6" max="6" width="59.1796875" customWidth="1"/>
-    <col min="7" max="7" width="31.453125" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" customWidth="1"/>
-    <col min="9" max="9" width="59.1796875" customWidth="1"/>
-    <col min="10" max="10" width="31.453125" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" customWidth="1"/>
-    <col min="12" max="12" width="23.81640625" customWidth="1"/>
-    <col min="13" max="14" width="11.453125" customWidth="1"/>
-    <col min="15" max="15" width="17.81640625" customWidth="1"/>
-    <col min="16" max="16" width="20.1796875" customWidth="1"/>
-    <col min="17" max="26" width="11.453125" customWidth="1"/>
+    <col min="1" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="59.140625" customWidth="1"/>
+    <col min="7" max="7" width="31.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="59.140625" customWidth="1"/>
+    <col min="10" max="10" width="31.42578125" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="23.85546875" customWidth="1"/>
+    <col min="13" max="14" width="11.42578125" customWidth="1"/>
+    <col min="15" max="15" width="17.85546875" customWidth="1"/>
+    <col min="16" max="16" width="20.140625" customWidth="1"/>
+    <col min="17" max="26" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:16" ht="16">
+    <row r="3" spans="3:16" ht="15.75">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -9994,7 +9970,7 @@
       </c>
       <c r="L3" s="93"/>
     </row>
-    <row r="4" spans="3:16" ht="14.5">
+    <row r="4" spans="3:16">
       <c r="C4" s="1" t="s">
         <v>73</v>
       </c>
@@ -10019,7 +9995,7 @@
       <c r="O4" s="17"/>
       <c r="P4" s="18"/>
     </row>
-    <row r="5" spans="3:16" ht="14.5">
+    <row r="5" spans="3:16">
       <c r="C5" s="1" t="s">
         <v>75</v>
       </c>
@@ -10044,14 +10020,14 @@
       <c r="O5" s="16"/>
       <c r="P5" s="19"/>
     </row>
-    <row r="6" spans="3:16" ht="14.5">
+    <row r="6" spans="3:16">
       <c r="L6" s="3"/>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
       <c r="P6" s="19"/>
     </row>
-    <row r="7" spans="3:16" ht="14.5">
+    <row r="7" spans="3:16">
       <c r="C7" s="1" t="s">
         <v>77</v>
       </c>
@@ -10079,7 +10055,7 @@
       <c r="O7" s="22"/>
       <c r="P7" s="19"/>
     </row>
-    <row r="8" spans="3:16" ht="14.5">
+    <row r="8" spans="3:16">
       <c r="C8" s="1" t="s">
         <v>118</v>
       </c>
@@ -10105,7 +10081,7 @@
       <c r="O8" s="24"/>
       <c r="P8" s="19"/>
     </row>
-    <row r="9" spans="3:16" ht="14.5">
+    <row r="9" spans="3:16">
       <c r="C9" s="1" t="s">
         <v>119</v>
       </c>
@@ -10133,7 +10109,7 @@
       <c r="O9" s="16"/>
       <c r="P9" s="19"/>
     </row>
-    <row r="10" spans="3:16" ht="14.5">
+    <row r="10" spans="3:16">
       <c r="C10" s="1" t="s">
         <v>84</v>
       </c>
@@ -10152,7 +10128,7 @@
       <c r="O10" s="3"/>
       <c r="P10" s="19"/>
     </row>
-    <row r="12" spans="3:16" ht="14.5">
+    <row r="12" spans="3:16">
       <c r="C12" s="1" t="s">
         <v>86</v>
       </c>
@@ -10166,7 +10142,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="13" spans="3:16" ht="14.5">
+    <row r="13" spans="3:16">
       <c r="C13" s="1" t="s">
         <v>88</v>
       </c>
@@ -10180,7 +10156,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="3:16" ht="14.5">
+    <row r="14" spans="3:16">
       <c r="C14" s="1" t="s">
         <v>90</v>
       </c>
@@ -10194,7 +10170,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="3:16" ht="14.5">
+    <row r="15" spans="3:16">
       <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
@@ -10217,7 +10193,7 @@
         <v>4.2588727636363641</v>
       </c>
     </row>
-    <row r="19" spans="3:10" ht="14.5">
+    <row r="19" spans="3:10">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -10228,7 +10204,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:10" ht="14.5">
+    <row r="20" spans="3:10">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -11852,36 +11828,36 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="C2:X1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.453125" customWidth="1"/>
-    <col min="3" max="3" width="58.54296875" customWidth="1"/>
-    <col min="4" max="4" width="30.1796875" customWidth="1"/>
-    <col min="5" max="6" width="11.453125" customWidth="1"/>
+    <col min="1" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" customWidth="1"/>
-    <col min="9" max="10" width="11.453125" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" customWidth="1"/>
+    <col min="9" max="10" width="11.42578125" customWidth="1"/>
     <col min="11" max="11" width="59" customWidth="1"/>
-    <col min="12" max="12" width="13.453125" customWidth="1"/>
-    <col min="13" max="14" width="11.453125" customWidth="1"/>
-    <col min="15" max="15" width="26.54296875" customWidth="1"/>
-    <col min="16" max="17" width="11.81640625" customWidth="1"/>
-    <col min="18" max="18" width="16.7265625" customWidth="1"/>
-    <col min="19" max="19" width="11.453125" customWidth="1"/>
-    <col min="20" max="20" width="22.54296875" customWidth="1"/>
-    <col min="21" max="23" width="11.453125" customWidth="1"/>
-    <col min="24" max="24" width="14.1796875" customWidth="1"/>
-    <col min="25" max="33" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="13" max="14" width="11.42578125" customWidth="1"/>
+    <col min="15" max="15" width="26.5703125" customWidth="1"/>
+    <col min="16" max="17" width="11.85546875" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" customWidth="1"/>
+    <col min="19" max="19" width="11.42578125" customWidth="1"/>
+    <col min="20" max="20" width="22.5703125" customWidth="1"/>
+    <col min="21" max="23" width="11.42578125" customWidth="1"/>
+    <col min="24" max="24" width="14.140625" customWidth="1"/>
+    <col min="25" max="33" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:24" ht="14.5">
+    <row r="2" spans="3:24">
       <c r="T2" s="16"/>
       <c r="U2" s="17"/>
       <c r="V2" s="17"/>
       <c r="W2" s="17"/>
       <c r="X2" s="18"/>
     </row>
-    <row r="3" spans="3:24" ht="14.5">
+    <row r="3" spans="3:24">
       <c r="C3" s="5" t="s">
         <v>66</v>
       </c>
@@ -11910,7 +11886,7 @@
       <c r="W3" s="16"/>
       <c r="X3" s="19"/>
     </row>
-    <row r="4" spans="3:24" ht="14.5">
+    <row r="4" spans="3:24">
       <c r="C4" s="5" t="s">
         <v>73</v>
       </c>
@@ -11939,7 +11915,7 @@
       <c r="W4" s="16"/>
       <c r="X4" s="19"/>
     </row>
-    <row r="5" spans="3:24" ht="14.5">
+    <row r="5" spans="3:24">
       <c r="C5" s="3" t="s">
         <v>75</v>
       </c>
@@ -11968,7 +11944,7 @@
       <c r="W5" s="22"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="3:24" ht="14.5">
+    <row r="6" spans="3:24">
       <c r="O6" s="16"/>
       <c r="P6" s="21"/>
       <c r="Q6" s="21"/>
@@ -11979,7 +11955,7 @@
       <c r="W6" s="24"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="3:24" ht="14.5">
+    <row r="7" spans="3:24">
       <c r="C7" s="1" t="s">
         <v>77</v>
       </c>
@@ -12009,7 +11985,7 @@
       <c r="W7" s="16"/>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="3:24" ht="14.5">
+    <row r="8" spans="3:24">
       <c r="C8" s="1" t="s">
         <v>79</v>
       </c>
@@ -12033,7 +12009,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
     </row>
-    <row r="9" spans="3:24" ht="14.5">
+    <row r="9" spans="3:24">
       <c r="C9" s="1" t="s">
         <v>81</v>
       </c>
@@ -12041,7 +12017,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="3:24" ht="14.5">
+    <row r="10" spans="3:24">
       <c r="C10" s="1" t="s">
         <v>82</v>
       </c>
@@ -12050,7 +12026,7 @@
         <v>87.3</v>
       </c>
     </row>
-    <row r="11" spans="3:24" ht="14.5">
+    <row r="11" spans="3:24">
       <c r="C11" s="1" t="s">
         <v>83</v>
       </c>
@@ -12075,7 +12051,7 @@
       </c>
       <c r="P11" s="97"/>
     </row>
-    <row r="12" spans="3:24" ht="14.5">
+    <row r="12" spans="3:24">
       <c r="C12" s="1" t="s">
         <v>86</v>
       </c>
@@ -12101,7 +12077,7 @@
         <v>5957</v>
       </c>
     </row>
-    <row r="13" spans="3:24" ht="14.5">
+    <row r="13" spans="3:24">
       <c r="C13" s="1" t="s">
         <v>88</v>
       </c>
@@ -12127,7 +12103,7 @@
         <v>2286</v>
       </c>
     </row>
-    <row r="14" spans="3:24" ht="14.5">
+    <row r="14" spans="3:24">
       <c r="C14" s="1" t="s">
         <v>90</v>
       </c>
@@ -12153,7 +12129,7 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="15" spans="3:24" ht="14.5">
+    <row r="15" spans="3:24">
       <c r="C15" s="1" t="s">
         <v>92</v>
       </c>
@@ -12183,7 +12159,7 @@
         <v>33962548788</v>
       </c>
     </row>
-    <row r="16" spans="3:24" ht="14.5">
+    <row r="16" spans="3:24">
       <c r="O16" s="16" t="s">
         <v>95</v>
       </c>
@@ -12191,7 +12167,7 @@
         <v>33.963000000000001</v>
       </c>
     </row>
-    <row r="17" spans="3:17" ht="14.5">
+    <row r="17" spans="3:17">
       <c r="O17" s="17" t="s">
         <v>96</v>
       </c>
@@ -12199,7 +12175,7 @@
         <v>33963</v>
       </c>
     </row>
-    <row r="18" spans="3:17" ht="14.5">
+    <row r="18" spans="3:17">
       <c r="O18" s="17" t="s">
         <v>97</v>
       </c>
@@ -12207,7 +12183,7 @@
         <v>13750</v>
       </c>
     </row>
-    <row r="19" spans="3:17" ht="14.5">
+    <row r="19" spans="3:17">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -12218,7 +12194,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:17" ht="14.5">
+    <row r="20" spans="3:17">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -13898,33 +13874,33 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="C2:X1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="11.453125" customWidth="1"/>
-    <col min="3" max="3" width="58.54296875" customWidth="1"/>
-    <col min="4" max="4" width="30.1796875" customWidth="1"/>
-    <col min="5" max="6" width="11.453125" customWidth="1"/>
+    <col min="1" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" customWidth="1"/>
-    <col min="9" max="10" width="11.453125" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="10" width="11.42578125" customWidth="1"/>
     <col min="11" max="11" width="59" customWidth="1"/>
-    <col min="12" max="12" width="24.54296875" customWidth="1"/>
-    <col min="13" max="14" width="11.453125" customWidth="1"/>
-    <col min="15" max="15" width="22.54296875" customWidth="1"/>
-    <col min="16" max="17" width="11.81640625" customWidth="1"/>
-    <col min="18" max="18" width="16.7265625" customWidth="1"/>
-    <col min="19" max="19" width="11.453125" customWidth="1"/>
-    <col min="20" max="20" width="21.453125" customWidth="1"/>
-    <col min="21" max="22" width="11.453125" customWidth="1"/>
-    <col min="23" max="23" width="12.26953125" customWidth="1"/>
-    <col min="24" max="24" width="14.7265625" customWidth="1"/>
-    <col min="25" max="32" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="24.5703125" customWidth="1"/>
+    <col min="13" max="14" width="11.42578125" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" customWidth="1"/>
+    <col min="16" max="17" width="11.85546875" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" customWidth="1"/>
+    <col min="19" max="19" width="11.42578125" customWidth="1"/>
+    <col min="20" max="20" width="21.42578125" customWidth="1"/>
+    <col min="21" max="22" width="11.42578125" customWidth="1"/>
+    <col min="23" max="23" width="12.28515625" customWidth="1"/>
+    <col min="24" max="24" width="14.7109375" customWidth="1"/>
+    <col min="25" max="32" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:24" ht="16">
+    <row r="2" spans="3:24" ht="15.75">
       <c r="T2" s="93"/>
     </row>
-    <row r="3" spans="3:24" ht="14.5">
+    <row r="3" spans="3:24">
       <c r="C3" s="5" t="s">
         <v>66</v>
       </c>
@@ -13953,7 +13929,7 @@
       <c r="W3" s="17"/>
       <c r="X3" s="18"/>
     </row>
-    <row r="4" spans="3:24" ht="14.5">
+    <row r="4" spans="3:24">
       <c r="C4" s="5" t="s">
         <v>73</v>
       </c>
@@ -13982,7 +13958,7 @@
       <c r="W4" s="3"/>
       <c r="X4" s="19"/>
     </row>
-    <row r="5" spans="3:24" ht="14.5">
+    <row r="5" spans="3:24">
       <c r="C5" s="3" t="s">
         <v>75</v>
       </c>
@@ -14011,7 +13987,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="3:24" ht="14.5">
+    <row r="6" spans="3:24">
       <c r="K6" s="1" t="s">
         <v>119</v>
       </c>
@@ -14029,7 +14005,7 @@
       <c r="W6" s="20"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="3:24" ht="14.5">
+    <row r="7" spans="3:24">
       <c r="C7" s="1" t="s">
         <v>119</v>
       </c>
@@ -14059,7 +14035,7 @@
       <c r="W7" s="21"/>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="3:24" ht="14.5">
+    <row r="8" spans="3:24">
       <c r="C8" s="1" t="s">
         <v>118</v>
       </c>
@@ -14088,7 +14064,7 @@
       <c r="W8" s="3"/>
       <c r="X8" s="19"/>
     </row>
-    <row r="9" spans="3:24" ht="14.5">
+    <row r="9" spans="3:24">
       <c r="C9" s="1" t="s">
         <v>77</v>
       </c>
@@ -14104,7 +14080,7 @@
         <v>28.000000000000007</v>
       </c>
     </row>
-    <row r="10" spans="3:24" ht="14.5">
+    <row r="10" spans="3:24">
       <c r="C10" s="1" t="s">
         <v>84</v>
       </c>
@@ -14119,7 +14095,7 @@
         <v>3.3600000000000005E-2</v>
       </c>
     </row>
-    <row r="11" spans="3:24" ht="14.5">
+    <row r="11" spans="3:24">
       <c r="K11" s="1" t="s">
         <v>84</v>
       </c>
@@ -14127,7 +14103,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="12" spans="3:24" ht="14.5">
+    <row r="12" spans="3:24">
       <c r="C12" s="1" t="s">
         <v>134</v>
       </c>
@@ -14148,7 +14124,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="13" spans="3:24" ht="14.5">
+    <row r="13" spans="3:24">
       <c r="C13" s="1" t="s">
         <v>136</v>
       </c>
@@ -14168,7 +14144,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="3:24" ht="14.5">
+    <row r="15" spans="3:24">
       <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
@@ -14191,7 +14167,7 @@
         <v>1.69100936968451E-2</v>
       </c>
     </row>
-    <row r="19" spans="3:12" ht="14.5">
+    <row r="19" spans="3:12">
       <c r="C19" s="1" t="s">
         <v>66</v>
       </c>
@@ -14202,7 +14178,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="3:12" ht="14.5">
+    <row r="20" spans="3:12">
       <c r="C20" s="81" t="s">
         <v>34</v>
       </c>
@@ -15853,35 +15829,35 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="C3:AJ1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="10.54296875" customWidth="1"/>
-    <col min="3" max="3" width="25.453125" customWidth="1"/>
-    <col min="4" max="5" width="10.54296875" customWidth="1"/>
+    <col min="1" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" customWidth="1"/>
+    <col min="4" max="5" width="10.5703125" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="10" width="10.54296875" customWidth="1"/>
-    <col min="11" max="11" width="22.7265625" customWidth="1"/>
-    <col min="12" max="12" width="14.54296875" customWidth="1"/>
-    <col min="13" max="13" width="15.54296875" customWidth="1"/>
-    <col min="14" max="14" width="13.54296875" customWidth="1"/>
-    <col min="15" max="15" width="14.54296875" customWidth="1"/>
-    <col min="16" max="18" width="10.54296875" customWidth="1"/>
-    <col min="19" max="19" width="22.7265625" customWidth="1"/>
-    <col min="20" max="20" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="15" max="15" width="14.5703125" customWidth="1"/>
+    <col min="16" max="18" width="10.5703125" customWidth="1"/>
+    <col min="19" max="19" width="22.7109375" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="13" customWidth="1"/>
-    <col min="24" max="26" width="10.54296875" customWidth="1"/>
-    <col min="27" max="27" width="22.7265625" customWidth="1"/>
-    <col min="28" max="28" width="8.26953125" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" customWidth="1"/>
-    <col min="30" max="30" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.26953125" customWidth="1"/>
-    <col min="32" max="32" width="10.54296875" customWidth="1"/>
-    <col min="33" max="33" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" customWidth="1"/>
+    <col min="24" max="26" width="10.5703125" customWidth="1"/>
+    <col min="27" max="27" width="22.7109375" customWidth="1"/>
+    <col min="28" max="28" width="8.28515625" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" customWidth="1"/>
+    <col min="30" max="30" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.28515625" customWidth="1"/>
+    <col min="32" max="32" width="10.5703125" customWidth="1"/>
+    <col min="33" max="33" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:36" ht="14.5">
+    <row r="3" spans="3:36">
       <c r="C3" s="105" t="s">
         <v>110</v>
       </c>
@@ -15917,7 +15893,7 @@
       <c r="AI3" s="106"/>
       <c r="AJ3" s="107"/>
     </row>
-    <row r="4" spans="3:36" ht="14.5">
+    <row r="4" spans="3:36">
       <c r="C4" s="35"/>
       <c r="D4" s="36" t="s">
         <v>113</v>
@@ -15981,7 +15957,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="3:36" ht="14.5">
+    <row r="5" spans="3:36">
       <c r="C5" s="35" t="s">
         <v>74</v>
       </c>
@@ -16031,7 +16007,7 @@
         <v>13333.333333333334</v>
       </c>
       <c r="AA5" s="35" t="s">
-        <v>74</v>
+        <v>179</v>
       </c>
       <c r="AB5" s="39">
         <v>1333.3333333333333</v>
@@ -16047,7 +16023,7 @@
         <v>5722.2222222222226</v>
       </c>
       <c r="AG5" s="35" t="s">
-        <v>74</v>
+        <v>179</v>
       </c>
       <c r="AH5" s="39">
         <v>1333.3333333333333</v>
@@ -16060,7 +16036,7 @@
         <v>1916.6666666666665</v>
       </c>
     </row>
-    <row r="6" spans="3:36" ht="14.5">
+    <row r="6" spans="3:36">
       <c r="C6" s="35" t="s">
         <v>117</v>
       </c>
@@ -16119,7 +16095,7 @@
         <v>30629805.333333332</v>
       </c>
       <c r="AA6" s="35" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="AB6" s="39">
         <v>12595</v>
@@ -16135,7 +16111,7 @@
         <v>10217999.555555554</v>
       </c>
       <c r="AG6" s="35" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="AH6" s="92">
         <v>12595</v>
@@ -16148,7 +16124,7 @@
         <v>12096.666666666668</v>
       </c>
     </row>
-    <row r="7" spans="3:36" ht="14.5">
+    <row r="7" spans="3:36">
       <c r="C7" s="35" t="s">
         <v>118</v>
       </c>
@@ -16236,7 +16212,7 @@
         <v>20389.349999999999</v>
       </c>
     </row>
-    <row r="8" spans="3:36" ht="14.5">
+    <row r="8" spans="3:36">
       <c r="C8" s="35" t="s">
         <v>92</v>
       </c>
@@ -16324,7 +16300,7 @@
         <v>19.444272973333334</v>
       </c>
     </row>
-    <row r="9" spans="3:36" ht="14.5">
+    <row r="9" spans="3:36">
       <c r="C9" s="35" t="s">
         <v>78</v>
       </c>
@@ -16412,7 +16388,7 @@
         <v>2940.625</v>
       </c>
     </row>
-    <row r="13" spans="3:36" ht="14.5">
+    <row r="13" spans="3:36">
       <c r="C13" s="105" t="s">
         <v>138</v>
       </c>
@@ -16448,7 +16424,7 @@
       <c r="AI13" s="106"/>
       <c r="AJ13" s="107"/>
     </row>
-    <row r="14" spans="3:36" ht="14.5">
+    <row r="14" spans="3:36">
       <c r="C14" s="35"/>
       <c r="D14" s="36" t="s">
         <v>113</v>
@@ -16512,7 +16488,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="3:36" ht="14.5">
+    <row r="15" spans="3:36">
       <c r="C15" s="35" t="s">
         <v>74</v>
       </c>
@@ -16571,7 +16547,7 @@
         <v>0.66666666666666674</v>
       </c>
       <c r="AA15" s="35" t="s">
-        <v>74</v>
+        <v>179</v>
       </c>
       <c r="AB15" s="40">
         <f>AB5/$AD$5</f>
@@ -16585,12 +16561,9 @@
         <f t="shared" si="8"/>
         <v>1</v>
       </c>
-      <c r="AE15" s="40">
-        <f t="shared" si="8"/>
-        <v>0.4291666666666667</v>
-      </c>
+      <c r="AE15" s="40"/>
       <c r="AG15" s="35" t="s">
-        <v>74</v>
+        <v>179</v>
       </c>
       <c r="AH15" s="40">
         <f>AH5/$AI$5</f>
@@ -16600,12 +16573,9 @@
         <f t="shared" ref="AI15:AJ15" si="9">AI5/$AI$5</f>
         <v>1</v>
       </c>
-      <c r="AJ15" s="40">
-        <f t="shared" si="9"/>
-        <v>0.76666666666666661</v>
-      </c>
-    </row>
-    <row r="16" spans="3:36" ht="14.5">
+      <c r="AJ15" s="40"/>
+    </row>
+    <row r="16" spans="3:36">
       <c r="C16" s="35" t="s">
         <v>117</v>
       </c>
@@ -16664,7 +16634,7 @@
         <v>0.36755722440155958</v>
       </c>
       <c r="AA16" s="35" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="AB16" s="40">
         <f>AB6/$AD$6</f>
@@ -16678,12 +16648,9 @@
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="AE16" s="40">
-        <f t="shared" si="13"/>
-        <v>0.33359662081938429</v>
-      </c>
+      <c r="AE16" s="40"/>
       <c r="AG16" s="35" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="AH16" s="92">
         <f>AH6/$AH$6</f>
@@ -16693,12 +16660,9 @@
         <f t="shared" ref="AI16:AJ16" si="14">AI6/$AH$6</f>
         <v>0.92086806933968512</v>
       </c>
-      <c r="AJ16" s="40">
-        <f t="shared" si="14"/>
-        <v>0.96043403466984267</v>
-      </c>
-    </row>
-    <row r="17" spans="3:36" ht="14.5">
+      <c r="AJ16" s="40"/>
+    </row>
+    <row r="17" spans="3:36">
       <c r="C17" s="35" t="s">
         <v>118</v>
       </c>
@@ -16771,10 +16735,7 @@
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="AE17" s="40">
-        <f t="shared" si="18"/>
-        <v>0.38212279811629662</v>
-      </c>
+      <c r="AE17" s="40"/>
       <c r="AG17" s="35" t="s">
         <v>118</v>
       </c>
@@ -16786,12 +16747,9 @@
         <f t="shared" ref="AI17:AJ17" si="19">AI7/$AI$7</f>
         <v>1</v>
       </c>
-      <c r="AJ17" s="40">
-        <f t="shared" si="19"/>
-        <v>0.72741602697126273</v>
-      </c>
-    </row>
-    <row r="18" spans="3:36" ht="14.5">
+      <c r="AJ17" s="40"/>
+    </row>
+    <row r="18" spans="3:36">
       <c r="C18" s="35" t="s">
         <v>92</v>
       </c>
@@ -16864,10 +16822,7 @@
         <f t="shared" si="23"/>
         <v>1</v>
       </c>
-      <c r="AE18" s="40">
-        <f t="shared" si="23"/>
-        <v>0.44179055316397275</v>
-      </c>
+      <c r="AE18" s="40"/>
       <c r="AG18" s="35" t="s">
         <v>92</v>
       </c>
@@ -16879,12 +16834,9 @@
         <f t="shared" ref="AI18:AJ18" si="24">AI8/$AI$8</f>
         <v>1</v>
       </c>
-      <c r="AJ18" s="40">
-        <f t="shared" si="24"/>
-        <v>0.85406533109231642</v>
-      </c>
-    </row>
-    <row r="19" spans="3:36" ht="14.5">
+      <c r="AJ18" s="40"/>
+    </row>
+    <row r="19" spans="3:36">
       <c r="C19" s="35" t="s">
         <v>78</v>
       </c>
@@ -16957,10 +16909,7 @@
         <f t="shared" si="28"/>
         <v>0.62099572881355936</v>
       </c>
-      <c r="AE19" s="40">
-        <f t="shared" si="28"/>
-        <v>0.73863699435028241</v>
-      </c>
+      <c r="AE19" s="40"/>
       <c r="AG19" s="35" t="s">
         <v>78</v>
       </c>
@@ -16972,10 +16921,7 @@
         <f t="shared" ref="AI19:AJ19" si="29">AI9/$AI$9</f>
         <v>1</v>
       </c>
-      <c r="AJ19" s="40">
-        <f t="shared" si="29"/>
-        <v>0.7974576271186441</v>
-      </c>
+      <c r="AJ19" s="40"/>
     </row>
     <row r="21" spans="3:36" ht="15.75" customHeight="1"/>
     <row r="22" spans="3:36" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
:white_circle: Dev v5.2: CH5 - Batt Bank simulations
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4B5879-BC75-4816-A9C6-30D58F219F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3A50749-8C77-4608-9C2C-47116DB3F884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
@@ -5954,6 +5954,10 @@
         <f t="shared" si="1"/>
         <v>91.25</v>
       </c>
+      <c r="G9">
+        <f>(E9*1000)/780</f>
+        <v>233.97435897435898</v>
+      </c>
       <c r="H9" s="42"/>
       <c r="I9" s="43"/>
       <c r="J9" s="42"/>
@@ -6200,7 +6204,14 @@
         <f t="shared" ref="F21:F27" si="2">E21*$B$7</f>
         <v>273.75</v>
       </c>
-      <c r="H21" s="42"/>
+      <c r="G21">
+        <f>(E21*1000)/780</f>
+        <v>701.92307692307691</v>
+      </c>
+      <c r="H21" s="42">
+        <f>G21-G9</f>
+        <v>467.9487179487179</v>
+      </c>
       <c r="I21" s="70"/>
       <c r="J21" s="42"/>
       <c r="K21" s="42"/>
@@ -6240,7 +6251,14 @@
         <f t="shared" si="2"/>
         <v>182.5</v>
       </c>
-      <c r="H23" s="42"/>
+      <c r="G23">
+        <f>(E23*1000)/780</f>
+        <v>467.94871794871796</v>
+      </c>
+      <c r="H23" s="42">
+        <f>G23-G21</f>
+        <v>-233.97435897435895</v>
+      </c>
       <c r="I23" s="70"/>
       <c r="J23" s="42"/>
       <c r="K23" s="42"/>
@@ -6689,7 +6707,10 @@
         <f t="shared" ref="F5:F24" si="1">$B$4*E5</f>
         <v>182.5</v>
       </c>
-      <c r="G5" s="42"/>
+      <c r="G5" s="42">
+        <f>(E5*1000)/780</f>
+        <v>467.94871794871796</v>
+      </c>
       <c r="H5" s="42"/>
       <c r="I5" s="42"/>
       <c r="K5" s="42"/>
@@ -6853,8 +6874,14 @@
         <f t="shared" si="1"/>
         <v>273.75</v>
       </c>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
+      <c r="G11" s="42">
+        <f>(E11*1000)/780</f>
+        <v>701.92307692307691</v>
+      </c>
+      <c r="H11" s="42">
+        <f>G11-G5</f>
+        <v>233.97435897435895</v>
+      </c>
       <c r="I11" s="42"/>
       <c r="K11" s="42"/>
       <c r="L11" s="42"/>
@@ -6881,8 +6908,14 @@
         <f t="shared" si="1"/>
         <v>91.25</v>
       </c>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
+      <c r="G12" s="42">
+        <f>(E12*1000)/780</f>
+        <v>233.97435897435898</v>
+      </c>
+      <c r="H12" s="42">
+        <f>G12-G11</f>
+        <v>-467.9487179487179</v>
+      </c>
       <c r="I12" s="42"/>
       <c r="K12" s="42"/>
       <c r="L12" s="42"/>
@@ -16554,7 +16587,7 @@
         <v>9.9999999999999992E-2</v>
       </c>
       <c r="AC15" s="40">
-        <f t="shared" ref="AC15:AE15" si="8">AC5/$AD$5</f>
+        <f t="shared" ref="AC15:AD15" si="8">AC5/$AD$5</f>
         <v>0.1875</v>
       </c>
       <c r="AD15" s="92">
@@ -16570,7 +16603,7 @@
         <v>0.53333333333333333</v>
       </c>
       <c r="AI15" s="92">
-        <f t="shared" ref="AI15:AJ15" si="9">AI5/$AI$5</f>
+        <f t="shared" ref="AI15" si="9">AI5/$AI$5</f>
         <v>1</v>
       </c>
       <c r="AJ15" s="40"/>
@@ -16641,7 +16674,7 @@
         <v>4.1120078508279995E-4</v>
       </c>
       <c r="AC16" s="40">
-        <f t="shared" ref="AC16:AE16" si="13">AC6/$AD$6</f>
+        <f t="shared" ref="AC16:AD16" si="13">AC6/$AD$6</f>
         <v>3.7866167307016083E-4</v>
       </c>
       <c r="AD16" s="92">
@@ -16657,7 +16690,7 @@
         <v>1</v>
       </c>
       <c r="AI16" s="40">
-        <f t="shared" ref="AI16:AJ16" si="14">AI6/$AH$6</f>
+        <f t="shared" ref="AI16" si="14">AI6/$AH$6</f>
         <v>0.92086806933968512</v>
       </c>
       <c r="AJ16" s="40"/>
@@ -16728,7 +16761,7 @@
         <v>4.5759946829302622E-2</v>
       </c>
       <c r="AC17" s="40">
-        <f t="shared" ref="AC17:AE17" si="18">AC7/$AD$7</f>
+        <f t="shared" ref="AC17:AD17" si="18">AC7/$AD$7</f>
         <v>0.10060844751958715</v>
       </c>
       <c r="AD17" s="92">
@@ -16744,7 +16777,7 @@
         <v>0.45483205394252563</v>
       </c>
       <c r="AI17" s="92">
-        <f t="shared" ref="AI17:AJ17" si="19">AI7/$AI$7</f>
+        <f t="shared" ref="AI17" si="19">AI7/$AI$7</f>
         <v>1</v>
       </c>
       <c r="AJ17" s="40"/>
@@ -16815,7 +16848,7 @@
         <v>0.13488760186380885</v>
       </c>
       <c r="AC18" s="40">
-        <f t="shared" ref="AC18:AE18" si="23">AC8/$AD$8</f>
+        <f t="shared" ref="AC18:AD18" si="23">AC8/$AD$8</f>
         <v>0.19048405762810935</v>
       </c>
       <c r="AD18" s="92">
@@ -16831,7 +16864,7 @@
         <v>0.70813066218463283</v>
       </c>
       <c r="AI18" s="92">
-        <f t="shared" ref="AI18:AJ18" si="24">AI8/$AI$8</f>
+        <f t="shared" ref="AI18" si="24">AI8/$AI$8</f>
         <v>1</v>
       </c>
       <c r="AJ18" s="40"/>
@@ -16902,7 +16935,7 @@
         <v>0.59491525423728808</v>
       </c>
       <c r="AC19" s="92">
-        <f t="shared" ref="AC19:AE19" si="28">AC9/$AC$9</f>
+        <f t="shared" ref="AC19:AD19" si="28">AC9/$AC$9</f>
         <v>1</v>
       </c>
       <c r="AD19" s="40">
@@ -16918,7 +16951,7 @@
         <v>0.59491525423728808</v>
       </c>
       <c r="AI19" s="92">
-        <f t="shared" ref="AI19:AJ19" si="29">AI9/$AI$9</f>
+        <f t="shared" ref="AI19" si="29">AI9/$AI$9</f>
         <v>1</v>
       </c>
       <c r="AJ19" s="40"/>

</xml_diff>

<commit_message>
:white_circle: Dev v6.2.1: Tesis sin Agradecimientos
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/01_Diseño_banco_batt_015.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6008D82B-24EE-4A8B-8AA7-0BFC1F030281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FBA5857-8796-41B8-A8F9-DA96A2E0BEFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_15%" sheetId="8" r:id="rId1"/>
     <sheet name="2m_15%" sheetId="9" r:id="rId2"/>
     <sheet name="EnergyDemand_15%" sheetId="10" r:id="rId3"/>
     <sheet name="Batt3" sheetId="3" r:id="rId4"/>
-    <sheet name="NMC" sheetId="5" r:id="rId5"/>
-    <sheet name="LFP" sheetId="4" r:id="rId6"/>
+    <sheet name="LFP" sheetId="4" r:id="rId5"/>
+    <sheet name="NMC" sheetId="5" r:id="rId6"/>
     <sheet name="LTO" sheetId="6" r:id="rId7"/>
     <sheet name="Radar_Plot" sheetId="7" r:id="rId8"/>
   </sheets>
@@ -127,6 +127,69 @@
     <author/>
   </authors>
   <commentList>
+    <comment ref="C36" authorId="0" shapeId="0" xr:uid="{5E5CFAFA-CB9C-424F-AAB6-64ABE5E97BCA}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>======
+ID#AAABYWq4-HE
+Leonardo Solis Zamora    (2024-11-11 12:21:57)
+https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G36" authorId="0" shapeId="0" xr:uid="{94E34E4E-39A7-4F6A-B8BE-D3B46C47E4DD}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>======
+ID#AAABYWq4-HE
+Leonardo Solis Zamora    (2024-11-11 12:21:57)
+https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K36" authorId="0" shapeId="0" xr:uid="{575B06E8-573C-4782-BC14-4832BE57AF7C}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>======
+ID#AAABYWq4-HE
+Leonardo Solis Zamora    (2024-11-11 12:21:57)
+https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+  <extLst>
+    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miV9WjoyvENNABFJHeX9WU1rdnWOg=="/>
+    </ext>
+  </extLst>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
     <comment ref="C36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
       <text>
         <r>
@@ -179,69 +242,6 @@
   <extLst>
     <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhijWbr9bOGXsEHPF72CLOQVUVDKw=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C36" authorId="0" shapeId="0" xr:uid="{5E5CFAFA-CB9C-424F-AAB6-64ABE5E97BCA}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABYWq4-HE
-Leonardo Solis Zamora    (2024-11-11 12:21:57)
-https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G36" authorId="0" shapeId="0" xr:uid="{94E34E4E-39A7-4F6A-B8BE-D3B46C47E4DD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABYWq4-HE
-Leonardo Solis Zamora    (2024-11-11 12:21:57)
-https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K36" authorId="0" shapeId="0" xr:uid="{575B06E8-573C-4782-BC14-4832BE57AF7C}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABYWq4-HE
-Leonardo Solis Zamora    (2024-11-11 12:21:57)
-https://www.ecolithiumbattery.com/battery-c-rating/#:~:text=So%20different%20material%20battery%20will,3C%20about%20LiFePO4%20prismatic%20battery.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miV9WjoyvENNABFJHeX9WU1rdnWOg=="/>
     </ext>
   </extLst>
 </comments>
@@ -1356,6 +1356,17 @@
     <xf numFmtId="1" fontId="9" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1378,17 +1389,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -5865,12 +5865,12 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:13" ht="18.5">
-      <c r="C5" s="95" t="s">
+      <c r="C5" s="100" t="s">
         <v>151</v>
       </c>
-      <c r="D5" s="95"/>
-      <c r="E5" s="95"/>
-      <c r="F5" s="95"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="100"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="42" t="s">
@@ -7834,14 +7834,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="14.5">
-      <c r="B1" s="98" t="s">
+      <c r="B1" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="100"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="105"/>
     </row>
     <row r="2" spans="2:13" ht="14.5">
       <c r="B2" s="1" t="s">
@@ -7853,24 +7853,24 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="14.5">
-      <c r="B3" s="101" t="s">
+      <c r="B3" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="97"/>
-      <c r="F3" s="101" t="s">
+      <c r="C3" s="102"/>
+      <c r="F3" s="106" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="97"/>
+      <c r="G3" s="102"/>
     </row>
     <row r="4" spans="2:13" ht="14.5">
-      <c r="B4" s="96" t="s">
+      <c r="B4" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="97"/>
-      <c r="F4" s="96" t="s">
+      <c r="C4" s="102"/>
+      <c r="F4" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="97"/>
+      <c r="G4" s="102"/>
     </row>
     <row r="5" spans="2:13" ht="14.5">
       <c r="B5" s="6" t="s">
@@ -7961,14 +7961,14 @@
       </c>
     </row>
     <row r="9" spans="2:13" ht="14.5">
-      <c r="B9" s="96" t="s">
+      <c r="B9" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="97"/>
-      <c r="F9" s="96" t="s">
+      <c r="C9" s="102"/>
+      <c r="F9" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="97"/>
+      <c r="G9" s="102"/>
       <c r="J9" s="1">
         <v>14</v>
       </c>
@@ -8125,10 +8125,10 @@
       </c>
     </row>
     <row r="15" spans="2:13" ht="14.5">
-      <c r="B15" s="96" t="s">
+      <c r="B15" s="101" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="97"/>
+      <c r="C15" s="102"/>
       <c r="F15" s="6" t="s">
         <v>6</v>
       </c>
@@ -8283,14 +8283,14 @@
       </c>
     </row>
     <row r="24" spans="2:13" ht="15.75" customHeight="1">
-      <c r="B24" s="96" t="s">
+      <c r="B24" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="97"/>
-      <c r="F24" s="96" t="s">
+      <c r="C24" s="102"/>
+      <c r="F24" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="97"/>
+      <c r="G24" s="102"/>
       <c r="J24" s="1">
         <v>12</v>
       </c>
@@ -8548,14 +8548,14 @@
       </c>
     </row>
     <row r="35" spans="2:13" ht="15.75" customHeight="1">
-      <c r="B35" s="98" t="s">
+      <c r="B35" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="99"/>
-      <c r="D35" s="99"/>
-      <c r="E35" s="99"/>
-      <c r="F35" s="99"/>
-      <c r="G35" s="100"/>
+      <c r="C35" s="104"/>
+      <c r="D35" s="104"/>
+      <c r="E35" s="104"/>
+      <c r="F35" s="104"/>
+      <c r="G35" s="105"/>
     </row>
     <row r="36" spans="2:13" ht="15.75" customHeight="1">
       <c r="D36" s="1" t="s">
@@ -8757,14 +8757,14 @@
       </c>
     </row>
     <row r="51" spans="2:12" ht="15.75" customHeight="1">
-      <c r="B51" s="98" t="s">
+      <c r="B51" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="C51" s="100"/>
-      <c r="F51" s="98" t="s">
+      <c r="C51" s="105"/>
+      <c r="F51" s="103" t="s">
         <v>49</v>
       </c>
-      <c r="G51" s="100"/>
+      <c r="G51" s="105"/>
     </row>
     <row r="52" spans="2:12" ht="15.75" customHeight="1">
       <c r="B52" s="1" t="s">
@@ -9936,6 +9936,12 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="B1:G1"/>
@@ -9943,12 +9949,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -9961,1904 +9961,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="C3:P1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
-  <cols>
-    <col min="1" max="2" width="11.453125" customWidth="1"/>
-    <col min="3" max="3" width="58.54296875" customWidth="1"/>
-    <col min="4" max="4" width="30.1796875" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" customWidth="1"/>
-    <col min="6" max="6" width="59.1796875" customWidth="1"/>
-    <col min="7" max="7" width="31.453125" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" customWidth="1"/>
-    <col min="9" max="9" width="59.1796875" customWidth="1"/>
-    <col min="10" max="10" width="31.453125" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" customWidth="1"/>
-    <col min="12" max="12" width="23.81640625" customWidth="1"/>
-    <col min="13" max="14" width="11.453125" customWidth="1"/>
-    <col min="15" max="15" width="17.81640625" customWidth="1"/>
-    <col min="16" max="16" width="20.1796875" customWidth="1"/>
-    <col min="17" max="26" width="11.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="3:16" ht="16">
-      <c r="C3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" t="s">
-        <v>108</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" t="s">
-        <v>109</v>
-      </c>
-      <c r="L3" s="93"/>
-    </row>
-    <row r="4" spans="3:16" ht="14.5">
-      <c r="C4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L4" s="16"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="18"/>
-    </row>
-    <row r="5" spans="3:16" ht="14.5">
-      <c r="C5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="19"/>
-    </row>
-    <row r="6" spans="3:16" ht="14.5">
-      <c r="L6" s="3"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="19"/>
-    </row>
-    <row r="7" spans="3:16" ht="14.5">
-      <c r="C7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="1">
-        <f>D10/D8</f>
-        <v>150</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G7" s="9">
-        <f>G10/G8</f>
-        <v>171.42857142857142</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J7" s="9">
-        <f>J23/J8</f>
-        <v>898.82278078269167</v>
-      </c>
-      <c r="L7" s="16"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="19"/>
-    </row>
-    <row r="8" spans="3:16" ht="14.5">
-      <c r="C8" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G8" s="1">
-        <v>2.1</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="J8" s="9">
-        <f>J31</f>
-        <v>0.4762121212121212</v>
-      </c>
-      <c r="L8" s="16"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
-      <c r="O8" s="24"/>
-      <c r="P8" s="19"/>
-    </row>
-    <row r="9" spans="3:16" ht="14.5">
-      <c r="C9" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="9">
-        <f>D10/D15</f>
-        <v>244.89795918367346</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="G9" s="9">
-        <f>G10/G15</f>
-        <v>319.43212067435672</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="J9" s="30">
-        <f>J23/J15</f>
-        <v>100.50319105209351</v>
-      </c>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="19"/>
-    </row>
-    <row r="10" spans="3:16" ht="14.5">
-      <c r="C10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" s="1">
-        <v>120</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G10" s="1">
-        <v>360</v>
-      </c>
-      <c r="L10" s="16"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="19"/>
-    </row>
-    <row r="12" spans="3:16" ht="14.5">
-      <c r="C12" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D12" s="1">
-        <v>100</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="1">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="13" spans="3:16" ht="14.5">
-      <c r="C13" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" s="1">
-        <v>70</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G13" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="3:16" ht="14.5">
-      <c r="C14" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="D14" s="1">
-        <v>70</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="3:16" ht="14.5">
-      <c r="C15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="1">
-        <f>1000*D12*D13*D14/1000000000</f>
-        <v>0.49</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G15" s="1">
-        <f>1000*G12*G13*G14/1000000000</f>
-        <v>1.127</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="J15" s="31">
-        <f>J33*1000</f>
-        <v>4.2588727636363641</v>
-      </c>
-    </row>
-    <row r="19" spans="3:10" ht="14.5">
-      <c r="C19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="20" spans="3:10" ht="14.5">
-      <c r="C20" s="81" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="81">
-        <v>750</v>
-      </c>
-      <c r="F20" s="81" t="s">
-        <v>34</v>
-      </c>
-      <c r="G20" s="81">
-        <v>750</v>
-      </c>
-      <c r="I20" s="81" t="s">
-        <v>34</v>
-      </c>
-      <c r="J20" s="81">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="21" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C21" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" s="1">
-        <v>12</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G21" s="1">
-        <v>12</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J21" s="9">
-        <f>J20/J22</f>
-        <v>2.8409090909090908</v>
-      </c>
-    </row>
-    <row r="22" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C22" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="D22" s="1">
-        <f>ROUNDUP(D20/D21,0)</f>
-        <v>63</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="G22" s="1">
-        <f>ROUNDUP(G20/G21,0)</f>
-        <v>63</v>
-      </c>
-      <c r="I22" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="J22" s="1">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="23" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C23" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="1">
-        <f>D10</f>
-        <v>120</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G23" s="1">
-        <f>G10</f>
-        <v>360</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J23" s="4">
-        <f>J24/J22</f>
-        <v>428.030303030303</v>
-      </c>
-    </row>
-    <row r="24" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D24" s="1">
-        <f>D23*D22</f>
-        <v>7560</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G24" s="1">
-        <f>G23*G22</f>
-        <v>22680</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="J24" s="1">
-        <f>226000/2</f>
-        <v>113000</v>
-      </c>
-    </row>
-    <row r="25" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C25" s="81" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="81">
-        <v>2800000</v>
-      </c>
-      <c r="F25" s="81" t="s">
-        <v>39</v>
-      </c>
-      <c r="G25" s="81">
-        <v>2800000</v>
-      </c>
-      <c r="I25" s="81" t="s">
-        <v>39</v>
-      </c>
-      <c r="J25" s="81">
-        <v>2800000</v>
-      </c>
-    </row>
-    <row r="26" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C26" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="1">
-        <f>ROUNDUP(D25/D24,0)</f>
-        <v>371</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="G26" s="1">
-        <f>ROUNDUP(G25/G24,0)</f>
-        <v>124</v>
-      </c>
-      <c r="I26" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="J26" s="1">
-        <f>ROUNDUP(J25/J24,0)</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C27" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" s="1">
-        <v>10</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G27" s="1">
-        <v>30</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J27" s="1">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="28" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C28" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" s="1">
-        <f>D27*D26</f>
-        <v>3710</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G28" s="1">
-        <f>G27*G26</f>
-        <v>3720</v>
-      </c>
-      <c r="I28" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J28" s="1">
-        <f>J27*J26</f>
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="29" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C29" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="D29" s="1">
-        <f>D22*D26</f>
-        <v>23373</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="G29" s="1">
-        <f>G22*G26</f>
-        <v>7812</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="J29" s="1">
-        <f>J22*J26</f>
-        <v>6600</v>
-      </c>
-    </row>
-    <row r="30" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="31" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C31" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" s="1">
-        <f>D8</f>
-        <v>0.8</v>
-      </c>
-      <c r="F31" t="s">
-        <v>44</v>
-      </c>
-      <c r="G31" s="1">
-        <f>G8</f>
-        <v>2.1</v>
-      </c>
-      <c r="I31" t="s">
-        <v>44</v>
-      </c>
-      <c r="J31" s="9">
-        <f>J32/J29</f>
-        <v>0.4762121212121212</v>
-      </c>
-    </row>
-    <row r="32" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C32" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D32" s="1">
-        <f>D29*D31</f>
-        <v>18698.400000000001</v>
-      </c>
-      <c r="F32" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G32" s="1">
-        <f>G29*G31</f>
-        <v>16405.2</v>
-      </c>
-      <c r="I32" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="J32" s="1">
-        <v>3143</v>
-      </c>
-    </row>
-    <row r="33" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C33" t="s">
-        <v>177</v>
-      </c>
-      <c r="D33" s="94">
-        <f>D15/1000</f>
-        <v>4.8999999999999998E-4</v>
-      </c>
-      <c r="F33" t="s">
-        <v>177</v>
-      </c>
-      <c r="G33" s="1">
-        <f>G15/1000</f>
-        <v>1.127E-3</v>
-      </c>
-      <c r="I33" t="s">
-        <v>177</v>
-      </c>
-      <c r="J33" s="31">
-        <f>J34/J29</f>
-        <v>4.2588727636363637E-3</v>
-      </c>
-    </row>
-    <row r="34" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C34" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D34" s="1">
-        <f>D29*D33</f>
-        <v>11.452769999999999</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="G34" s="1">
-        <f>G29*G33</f>
-        <v>8.8041239999999998</v>
-      </c>
-      <c r="I34" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="J34" s="9">
-        <f>(1343*738*2836)/100000000</f>
-        <v>28.108560239999999</v>
-      </c>
-    </row>
-    <row r="35" spans="3:11" ht="15.75" customHeight="1"/>
-    <row r="36" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C36" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G36" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C37" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D37" s="1">
-        <v>1</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C38" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D38" s="1">
-        <v>3</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G38" s="1">
-        <v>3</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="J38" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C39" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="1">
-        <v>3</v>
-      </c>
-      <c r="F39" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="G39" s="1">
-        <v>5</v>
-      </c>
-      <c r="I39" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="J39" s="1">
-        <f>J27*J36</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="40" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C40" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="D40" s="1">
-        <v>5</v>
-      </c>
-      <c r="F40" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="G40" s="1">
-        <v>30</v>
-      </c>
-      <c r="I40" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="J40" s="1">
-        <f>J37*J27</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="41" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C41" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="D41" s="1">
-        <v>20</v>
-      </c>
-      <c r="F41" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="G41" s="1">
-        <v>60</v>
-      </c>
-      <c r="I41" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="J41" s="1">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="42" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C42" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" s="1">
-        <f>D41</f>
-        <v>20</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="G42" s="1">
-        <f>G41</f>
-        <v>60</v>
-      </c>
-      <c r="I42" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="J42" s="1">
-        <f>J41</f>
-        <v>750</v>
-      </c>
-    </row>
-    <row r="43" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C43" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D43" s="1">
-        <f>D42*D26</f>
-        <v>7420</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="G43" s="1">
-        <f>G42*G26</f>
-        <v>7440</v>
-      </c>
-      <c r="I43" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="J43" s="1">
-        <f>J42*J26</f>
-        <v>18750</v>
-      </c>
-    </row>
-    <row r="44" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C44" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D44" s="1">
-        <f>D43*D20</f>
-        <v>5565000</v>
-      </c>
-      <c r="E44">
-        <f>D44/1000</f>
-        <v>5565</v>
-      </c>
-      <c r="F44" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G44" s="1">
-        <f>G43*G20</f>
-        <v>5580000</v>
-      </c>
-      <c r="H44">
-        <f>G44/1000</f>
-        <v>5580</v>
-      </c>
-      <c r="I44" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="J44" s="1">
-        <f>J43*J20</f>
-        <v>14062500</v>
-      </c>
-      <c r="K44">
-        <f>J44/1000</f>
-        <v>14062.5</v>
-      </c>
-    </row>
-    <row r="45" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C45" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" s="1">
-        <f>D39</f>
-        <v>3</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="G45" s="1">
-        <f>G39</f>
-        <v>5</v>
-      </c>
-      <c r="I45" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="J45" s="1">
-        <f>J39</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="46" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C46" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D46" s="1">
-        <f>D45*D26</f>
-        <v>1113</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G46" s="1">
-        <f>G45*G26</f>
-        <v>620</v>
-      </c>
-      <c r="I46" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="J46" s="1">
-        <f>J45*J26</f>
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="47" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C47" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="D47" s="1">
-        <f>D46*D20</f>
-        <v>834750</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="G47" s="1">
-        <f>G46*G20</f>
-        <v>465000</v>
-      </c>
-      <c r="I47" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="J47" s="1">
-        <f>J46*J20</f>
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="48" spans="3:11" ht="15.75" customHeight="1">
-      <c r="C48" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="D48" s="1">
-        <v>5</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="G48" s="1">
-        <f>G40</f>
-        <v>30</v>
-      </c>
-      <c r="I48" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="J48" s="1">
-        <f>J40</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="49" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C49" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D49" s="1">
-        <f>D48*D26</f>
-        <v>1855</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G49" s="1">
-        <f>G48*G26</f>
-        <v>3720</v>
-      </c>
-      <c r="I49" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="J49" s="1">
-        <f>J48*J26</f>
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="50" spans="3:10" ht="15.75" customHeight="1">
-      <c r="C50" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D50" s="1">
-        <f>D49*D20/1000</f>
-        <v>1391.25</v>
-      </c>
-      <c r="F50" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G50" s="1">
-        <f>G49*G20/1000</f>
-        <v>2790</v>
-      </c>
-      <c r="I50" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="J50" s="1">
-        <f>J49*J20/1000</f>
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="51" spans="3:10" ht="15.75" customHeight="1">
-      <c r="D51">
-        <f>D50/1000</f>
-        <v>1.3912500000000001</v>
-      </c>
-      <c r="G51">
-        <f>G50/1000</f>
-        <v>2.79</v>
-      </c>
-      <c r="J51">
-        <f>J50/1000</f>
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="52" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="53" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="54" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="55" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="56" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="57" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="58" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="59" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="60" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="61" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="62" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="63" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="64" spans="3:10" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="C2:X1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
@@ -12079,10 +10181,10 @@
       <c r="L11" s="1">
         <v>1920</v>
       </c>
-      <c r="O11" s="102" t="s">
+      <c r="O11" s="107" t="s">
         <v>85</v>
       </c>
-      <c r="P11" s="97"/>
+      <c r="P11" s="102"/>
     </row>
     <row r="12" spans="3:24" ht="14.5">
       <c r="C12" s="1" t="s">
@@ -12246,10 +10348,10 @@
       <c r="L20" s="82">
         <v>750</v>
       </c>
-      <c r="O20" s="101" t="s">
+      <c r="O20" s="106" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="97"/>
+      <c r="P20" s="102"/>
     </row>
     <row r="21" spans="3:17" ht="15.75" customHeight="1">
       <c r="C21" s="1" t="s">
@@ -12358,10 +10460,10 @@
         <f>L23*L22</f>
         <v>38400</v>
       </c>
-      <c r="O24" s="103" t="s">
+      <c r="O24" s="108" t="s">
         <v>102</v>
       </c>
-      <c r="P24" s="97"/>
+      <c r="P24" s="102"/>
     </row>
     <row r="25" spans="3:17" ht="15.75" customHeight="1">
       <c r="C25" s="81" t="s">
@@ -12462,10 +10564,10 @@
         <f>L27*L26</f>
         <v>3650</v>
       </c>
-      <c r="O28" s="104" t="s">
+      <c r="O28" s="109" t="s">
         <v>147</v>
       </c>
-      <c r="P28" s="104"/>
+      <c r="P28" s="109"/>
     </row>
     <row r="29" spans="3:17" ht="15.75" customHeight="1">
       <c r="C29" s="14" t="s">
@@ -13901,6 +12003,1904 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="C3:P1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col min="1" max="2" width="11.453125" customWidth="1"/>
+    <col min="3" max="3" width="58.54296875" customWidth="1"/>
+    <col min="4" max="4" width="30.1796875" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="59.1796875" customWidth="1"/>
+    <col min="7" max="7" width="31.453125" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" customWidth="1"/>
+    <col min="9" max="9" width="59.1796875" customWidth="1"/>
+    <col min="10" max="10" width="31.453125" customWidth="1"/>
+    <col min="11" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="23.81640625" customWidth="1"/>
+    <col min="13" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="17.81640625" customWidth="1"/>
+    <col min="16" max="16" width="20.1796875" customWidth="1"/>
+    <col min="17" max="26" width="11.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:16" ht="16">
+      <c r="C3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" t="s">
+        <v>109</v>
+      </c>
+      <c r="L3" s="93"/>
+    </row>
+    <row r="4" spans="3:16" ht="14.5">
+      <c r="C4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="18"/>
+    </row>
+    <row r="5" spans="3:16" ht="14.5">
+      <c r="C5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="19"/>
+    </row>
+    <row r="6" spans="3:16" ht="14.5">
+      <c r="L6" s="3"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="19"/>
+    </row>
+    <row r="7" spans="3:16" ht="14.5">
+      <c r="C7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="1">
+        <f>D10/D8</f>
+        <v>150</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="9">
+        <f>G10/G8</f>
+        <v>171.42857142857142</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="9">
+        <f>J23/J8</f>
+        <v>898.82278078269167</v>
+      </c>
+      <c r="L7" s="16"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="19"/>
+    </row>
+    <row r="8" spans="3:16" ht="14.5">
+      <c r="C8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="J8" s="9">
+        <f>J31</f>
+        <v>0.4762121212121212</v>
+      </c>
+      <c r="L8" s="16"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="19"/>
+    </row>
+    <row r="9" spans="3:16" ht="14.5">
+      <c r="C9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D9" s="9">
+        <f>D10/D15</f>
+        <v>244.89795918367346</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G9" s="9">
+        <f>G10/G15</f>
+        <v>319.43212067435672</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J9" s="30">
+        <f>J23/J15</f>
+        <v>100.50319105209351</v>
+      </c>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="19"/>
+    </row>
+    <row r="10" spans="3:16" ht="14.5">
+      <c r="C10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="1">
+        <v>120</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="1">
+        <v>360</v>
+      </c>
+      <c r="L10" s="16"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="19"/>
+    </row>
+    <row r="12" spans="3:16" ht="14.5">
+      <c r="C12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="1">
+        <v>100</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G12" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="13" spans="3:16" ht="14.5">
+      <c r="C13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="1">
+        <v>70</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="3:16" ht="14.5">
+      <c r="C14" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D14" s="1">
+        <v>70</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="3:16" ht="14.5">
+      <c r="C15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="1">
+        <f>1000*D12*D13*D14/1000000000</f>
+        <v>0.49</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" s="1">
+        <f>1000*G12*G13*G14/1000000000</f>
+        <v>1.127</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" s="31">
+        <f>J33*1000</f>
+        <v>4.2588727636363641</v>
+      </c>
+    </row>
+    <row r="19" spans="3:10" ht="14.5">
+      <c r="C19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="3:10" ht="14.5">
+      <c r="C20" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="81">
+        <v>750</v>
+      </c>
+      <c r="F20" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="81">
+        <v>750</v>
+      </c>
+      <c r="I20" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="J20" s="81">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="21" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="1">
+        <v>12</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="1">
+        <v>12</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J21" s="9">
+        <f>J20/J22</f>
+        <v>2.8409090909090908</v>
+      </c>
+    </row>
+    <row r="22" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C22" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="D22" s="1">
+        <f>ROUNDUP(D20/D21,0)</f>
+        <v>63</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="G22" s="1">
+        <f>ROUNDUP(G20/G21,0)</f>
+        <v>63</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="J22" s="1">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="23" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="1">
+        <f>D10</f>
+        <v>120</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="1">
+        <f>G10</f>
+        <v>360</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J23" s="4">
+        <f>J24/J22</f>
+        <v>428.030303030303</v>
+      </c>
+    </row>
+    <row r="24" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="1">
+        <f>D23*D22</f>
+        <v>7560</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G24" s="1">
+        <f>G23*G22</f>
+        <v>22680</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="J24" s="1">
+        <f>226000/2</f>
+        <v>113000</v>
+      </c>
+    </row>
+    <row r="25" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C25" s="81" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="81">
+        <v>2800000</v>
+      </c>
+      <c r="F25" s="81" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" s="81">
+        <v>2800000</v>
+      </c>
+      <c r="I25" s="81" t="s">
+        <v>39</v>
+      </c>
+      <c r="J25" s="81">
+        <v>2800000</v>
+      </c>
+    </row>
+    <row r="26" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C26" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="1">
+        <f>ROUNDUP(D25/D24,0)</f>
+        <v>371</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G26" s="1">
+        <f>ROUNDUP(G25/G24,0)</f>
+        <v>124</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="J26" s="1">
+        <f>ROUNDUP(J25/J24,0)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" s="1">
+        <v>10</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G27" s="1">
+        <v>30</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J27" s="1">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="1">
+        <f>D27*D26</f>
+        <v>3710</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" s="1">
+        <f>G27*G26</f>
+        <v>3720</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="J28" s="1">
+        <f>J27*J26</f>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="29" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C29" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="D29" s="1">
+        <f>D22*D26</f>
+        <v>23373</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="G29" s="1">
+        <f>G22*G26</f>
+        <v>7812</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="J29" s="1">
+        <f>J22*J26</f>
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="30" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="31" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="1">
+        <f>D8</f>
+        <v>0.8</v>
+      </c>
+      <c r="F31" t="s">
+        <v>44</v>
+      </c>
+      <c r="G31" s="1">
+        <f>G8</f>
+        <v>2.1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>44</v>
+      </c>
+      <c r="J31" s="9">
+        <f>J32/J29</f>
+        <v>0.4762121212121212</v>
+      </c>
+    </row>
+    <row r="32" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D32" s="1">
+        <f>D29*D31</f>
+        <v>18698.400000000001</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G32" s="1">
+        <f>G29*G31</f>
+        <v>16405.2</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J32" s="1">
+        <v>3143</v>
+      </c>
+    </row>
+    <row r="33" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C33" t="s">
+        <v>177</v>
+      </c>
+      <c r="D33" s="94">
+        <f>D15/1000</f>
+        <v>4.8999999999999998E-4</v>
+      </c>
+      <c r="F33" t="s">
+        <v>177</v>
+      </c>
+      <c r="G33" s="1">
+        <f>G15/1000</f>
+        <v>1.127E-3</v>
+      </c>
+      <c r="I33" t="s">
+        <v>177</v>
+      </c>
+      <c r="J33" s="31">
+        <f>J34/J29</f>
+        <v>4.2588727636363637E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C34" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D34" s="1">
+        <f>D29*D33</f>
+        <v>11.452769999999999</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G34" s="1">
+        <f>G29*G33</f>
+        <v>8.8041239999999998</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="J34" s="9">
+        <f>(1343*738*2836)/100000000</f>
+        <v>28.108560239999999</v>
+      </c>
+    </row>
+    <row r="35" spans="3:11" ht="15.75" customHeight="1"/>
+    <row r="36" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G36" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J36" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C37" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" s="1">
+        <v>1</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G37" s="1">
+        <v>1</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C38" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="1">
+        <v>3</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G38" s="1">
+        <v>3</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J38" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C39" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" s="1">
+        <v>3</v>
+      </c>
+      <c r="F39" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="G39" s="1">
+        <v>5</v>
+      </c>
+      <c r="I39" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="J39" s="1">
+        <f>J27*J36</f>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C40" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="D40" s="1">
+        <v>5</v>
+      </c>
+      <c r="F40" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="G40" s="1">
+        <v>30</v>
+      </c>
+      <c r="I40" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="J40" s="1">
+        <f>J37*J27</f>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="41" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C41" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="D41" s="1">
+        <v>20</v>
+      </c>
+      <c r="F41" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G41" s="1">
+        <v>60</v>
+      </c>
+      <c r="I41" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="J41" s="1">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="42" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C42" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="1">
+        <f>D41</f>
+        <v>20</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G42" s="1">
+        <f>G41</f>
+        <v>60</v>
+      </c>
+      <c r="I42" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="J42" s="1">
+        <f>J41</f>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="43" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C43" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="1">
+        <f>D42*D26</f>
+        <v>7420</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G43" s="1">
+        <f>G42*G26</f>
+        <v>7440</v>
+      </c>
+      <c r="I43" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="J43" s="1">
+        <f>J42*J26</f>
+        <v>18750</v>
+      </c>
+    </row>
+    <row r="44" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C44" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D44" s="1">
+        <f>D43*D20</f>
+        <v>5565000</v>
+      </c>
+      <c r="E44">
+        <f>D44/1000</f>
+        <v>5565</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="G44" s="1">
+        <f>G43*G20</f>
+        <v>5580000</v>
+      </c>
+      <c r="H44">
+        <f>G44/1000</f>
+        <v>5580</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J44" s="1">
+        <f>J43*J20</f>
+        <v>14062500</v>
+      </c>
+      <c r="K44">
+        <f>J44/1000</f>
+        <v>14062.5</v>
+      </c>
+    </row>
+    <row r="45" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C45" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" s="1">
+        <f>D39</f>
+        <v>3</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G45" s="1">
+        <f>G39</f>
+        <v>5</v>
+      </c>
+      <c r="I45" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="J45" s="1">
+        <f>J39</f>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C46" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" s="1">
+        <f>D45*D26</f>
+        <v>1113</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G46" s="1">
+        <f>G45*G26</f>
+        <v>620</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="J46" s="1">
+        <f>J45*J26</f>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="47" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C47" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="1">
+        <f>D46*D20</f>
+        <v>834750</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G47" s="1">
+        <f>G46*G20</f>
+        <v>465000</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J47" s="1">
+        <f>J46*J20</f>
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="48" spans="3:11" ht="15.75" customHeight="1">
+      <c r="C48" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D48" s="1">
+        <v>5</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G48" s="1">
+        <f>G40</f>
+        <v>30</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J48" s="1">
+        <f>J40</f>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C49" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D49" s="1">
+        <f>D48*D26</f>
+        <v>1855</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G49" s="1">
+        <f>G48*G26</f>
+        <v>3720</v>
+      </c>
+      <c r="I49" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="J49" s="1">
+        <f>J48*J26</f>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="50" spans="3:10" ht="15.75" customHeight="1">
+      <c r="C50" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="1">
+        <f>D49*D20/1000</f>
+        <v>1391.25</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G50" s="1">
+        <f>G49*G20/1000</f>
+        <v>2790</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J50" s="1">
+        <f>J49*J20/1000</f>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="51" spans="3:10" ht="15.75" customHeight="1">
+      <c r="D51">
+        <f>D50/1000</f>
+        <v>1.3912500000000001</v>
+      </c>
+      <c r="G51">
+        <f>G50/1000</f>
+        <v>2.79</v>
+      </c>
+      <c r="J51">
+        <f>J50/1000</f>
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="52" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="53" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="54" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="55" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="56" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="57" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="58" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="59" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="60" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="61" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="62" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="63" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="64" spans="3:10" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15891,40 +15891,40 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:36" ht="14.5">
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="95" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="109"/>
-      <c r="K3" s="105" t="s">
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="99"/>
+      <c r="K3" s="95" t="s">
         <v>65</v>
       </c>
-      <c r="L3" s="106"/>
-      <c r="M3" s="106"/>
-      <c r="N3" s="106"/>
-      <c r="O3" s="107"/>
-      <c r="S3" s="105" t="s">
+      <c r="L3" s="96"/>
+      <c r="M3" s="96"/>
+      <c r="N3" s="96"/>
+      <c r="O3" s="97"/>
+      <c r="S3" s="95" t="s">
         <v>121</v>
       </c>
-      <c r="T3" s="106"/>
-      <c r="U3" s="106"/>
-      <c r="V3" s="106"/>
-      <c r="W3" s="107"/>
-      <c r="AA3" s="105" t="s">
+      <c r="T3" s="96"/>
+      <c r="U3" s="96"/>
+      <c r="V3" s="96"/>
+      <c r="W3" s="97"/>
+      <c r="AA3" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="AB3" s="106"/>
-      <c r="AC3" s="106"/>
-      <c r="AD3" s="106"/>
-      <c r="AE3" s="107"/>
-      <c r="AG3" s="105" t="s">
+      <c r="AB3" s="96"/>
+      <c r="AC3" s="96"/>
+      <c r="AD3" s="96"/>
+      <c r="AE3" s="97"/>
+      <c r="AG3" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="AH3" s="106"/>
-      <c r="AI3" s="106"/>
-      <c r="AJ3" s="107"/>
+      <c r="AH3" s="96"/>
+      <c r="AI3" s="96"/>
+      <c r="AJ3" s="97"/>
     </row>
     <row r="4" spans="3:36" ht="14.5">
       <c r="C4" s="35"/>
@@ -16422,40 +16422,40 @@
       </c>
     </row>
     <row r="13" spans="3:36" ht="14.5">
-      <c r="C13" s="105" t="s">
+      <c r="C13" s="95" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="106"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="106"/>
-      <c r="G13" s="107"/>
-      <c r="K13" s="105" t="s">
+      <c r="D13" s="96"/>
+      <c r="E13" s="96"/>
+      <c r="F13" s="96"/>
+      <c r="G13" s="97"/>
+      <c r="K13" s="95" t="s">
         <v>140</v>
       </c>
-      <c r="L13" s="106"/>
-      <c r="M13" s="106"/>
-      <c r="N13" s="106"/>
-      <c r="O13" s="107"/>
-      <c r="S13" s="105" t="s">
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="97"/>
+      <c r="S13" s="95" t="s">
         <v>139</v>
       </c>
-      <c r="T13" s="106"/>
-      <c r="U13" s="106"/>
-      <c r="V13" s="106"/>
-      <c r="W13" s="107"/>
-      <c r="AA13" s="105" t="s">
+      <c r="T13" s="96"/>
+      <c r="U13" s="96"/>
+      <c r="V13" s="96"/>
+      <c r="W13" s="97"/>
+      <c r="AA13" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="AB13" s="106"/>
-      <c r="AC13" s="106"/>
-      <c r="AD13" s="106"/>
-      <c r="AE13" s="107"/>
-      <c r="AG13" s="105" t="s">
+      <c r="AB13" s="96"/>
+      <c r="AC13" s="96"/>
+      <c r="AD13" s="96"/>
+      <c r="AE13" s="97"/>
+      <c r="AG13" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="AH13" s="106"/>
-      <c r="AI13" s="106"/>
-      <c r="AJ13" s="107"/>
+      <c r="AH13" s="96"/>
+      <c r="AI13" s="96"/>
+      <c r="AJ13" s="97"/>
     </row>
     <row r="14" spans="3:36" ht="14.5">
       <c r="C14" s="35"/>

</xml_diff>